<commit_message>
fixing the issue with too small or negative interrater agreement score. the correct values are are updated in the xlsx file
</commit_message>
<xml_diff>
--- a/data/annotations/TE_discrete_percentages.xlsx
+++ b/data/annotations/TE_discrete_percentages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\annotations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{BF42F981-D633-42A3-9A31-78C18F46FEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{FA16EFE5-F483-4B50-BE03-C341E916414E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{8450E3AB-A0C1-455F-AE9B-DBE7A60F6C99}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14856" activeTab="2" xr2:uid="{8450E3AB-A0C1-455F-AE9B-DBE7A60F6C99}"/>
   </bookViews>
   <sheets>
     <sheet name="TE_discrete_percentages" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="103">
   <si>
     <t>task_eng</t>
   </si>
@@ -322,6 +322,18 @@
   </si>
   <si>
     <t>dyads</t>
+  </si>
+  <si>
+    <t>.8 as top interval and then equal split</t>
+  </si>
+  <si>
+    <t xml:space="preserve">three way might be dificult to get good results; try also </t>
+  </si>
+  <si>
+    <t>Continous</t>
+  </si>
+  <si>
+    <t>Discrete</t>
   </si>
 </sst>
 </file>
@@ -32366,6 +32378,23 @@
         <v>0</v>
       </c>
     </row>
+    <row r="13" spans="1:108" x14ac:dyDescent="0.35">
+      <c r="BO13" t="s">
+        <v>52</v>
+      </c>
+      <c r="BP13" t="s">
+        <v>53</v>
+      </c>
+      <c r="BQ13" t="s">
+        <v>51</v>
+      </c>
+      <c r="BS13" t="s">
+        <v>52</v>
+      </c>
+      <c r="BT13" t="s">
+        <v>51</v>
+      </c>
+    </row>
     <row r="14" spans="1:108" x14ac:dyDescent="0.35">
       <c r="BI14" t="s">
         <v>71</v>
@@ -32378,6 +32407,21 @@
       </c>
       <c r="BL14" t="s">
         <v>70</v>
+      </c>
+      <c r="BO14">
+        <v>0.26600000000000001</v>
+      </c>
+      <c r="BP14">
+        <v>0.52600000000000002</v>
+      </c>
+      <c r="BQ14">
+        <v>0.78659999999999997</v>
+      </c>
+      <c r="BS14">
+        <v>0.4</v>
+      </c>
+      <c r="BT14">
+        <v>0.8</v>
       </c>
     </row>
     <row r="15" spans="1:108" x14ac:dyDescent="0.35">
@@ -32393,9 +32437,16 @@
       <c r="BL15" t="s">
         <v>67</v>
       </c>
+      <c r="BN15" s="2"/>
+      <c r="BO15" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="BS15" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="16" spans="1:108" x14ac:dyDescent="0.35">
-      <c r="BR16" t="s">
+      <c r="BR16" s="5" t="s">
         <v>64</v>
       </c>
     </row>
@@ -33329,7 +33380,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4135E192-98BF-45B4-BA3D-15FECDE552EF}">
-  <dimension ref="A1:AY9"/>
+  <dimension ref="A1:AY15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -33957,150 +34008,263 @@
         <v>0.27099410758410902</v>
       </c>
     </row>
-    <row r="6" spans="1:51" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" t="s">
-        <v>75</v>
-      </c>
-      <c r="E6" t="s">
-        <v>76</v>
-      </c>
-      <c r="F6" t="s">
-        <v>77</v>
-      </c>
-      <c r="G6" t="s">
-        <v>78</v>
-      </c>
-      <c r="H6" t="s">
-        <v>79</v>
-      </c>
-      <c r="I6" t="s">
-        <v>80</v>
-      </c>
-      <c r="J6" t="s">
-        <v>81</v>
-      </c>
-      <c r="K6" t="s">
-        <v>82</v>
-      </c>
-      <c r="L6" t="s">
-        <v>83</v>
-      </c>
-      <c r="M6" t="s">
-        <v>84</v>
-      </c>
-      <c r="N6" t="s">
-        <v>85</v>
-      </c>
-      <c r="O6" t="s">
-        <v>86</v>
-      </c>
-      <c r="P6" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>88</v>
-      </c>
-      <c r="R6" t="s">
-        <v>89</v>
-      </c>
-      <c r="S6" t="s">
-        <v>90</v>
-      </c>
-      <c r="T6" t="s">
-        <v>91</v>
-      </c>
-      <c r="U6" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="7" spans="1:51" x14ac:dyDescent="0.35">
-      <c r="B7">
-        <v>0.85629482756780495</v>
-      </c>
-      <c r="C7">
-        <v>0.72480082067718599</v>
-      </c>
-      <c r="D7">
-        <v>0.82777645880776596</v>
-      </c>
-      <c r="E7">
-        <v>0.82659452725981197</v>
-      </c>
-      <c r="F7">
-        <v>0.79078960048874103</v>
-      </c>
-      <c r="G7">
-        <v>0.83794847262402505</v>
-      </c>
-      <c r="H7">
-        <v>0.832584473541637</v>
-      </c>
-      <c r="I7">
-        <v>0.64171827186225805</v>
-      </c>
-      <c r="J7">
-        <v>0.86231599498596401</v>
-      </c>
-      <c r="K7">
-        <v>0.86957035714180098</v>
-      </c>
-      <c r="L7">
-        <v>0.53891218808139896</v>
-      </c>
-      <c r="M7">
-        <v>0.59137022905749004</v>
-      </c>
-      <c r="N7">
-        <v>0.44227699763089001</v>
-      </c>
-      <c r="P7">
-        <v>0.75878204633194901</v>
-      </c>
-      <c r="Q7">
-        <v>0.77646361437990297</v>
-      </c>
-      <c r="R7">
-        <v>0.57801020824920901</v>
-      </c>
-      <c r="S7">
-        <v>0.67676370745270498</v>
-      </c>
-      <c r="T7">
-        <v>0.61168228428765803</v>
-      </c>
-      <c r="U7">
-        <v>0.75541379016388399</v>
-      </c>
-    </row>
     <row r="8" spans="1:51" x14ac:dyDescent="0.35">
-      <c r="I8" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="U8" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="W8" s="5" t="s">
-        <v>96</v>
-      </c>
+      <c r="I8" s="5"/>
+      <c r="U8" s="5"/>
+      <c r="W8" s="5"/>
     </row>
     <row r="9" spans="1:51" x14ac:dyDescent="0.35">
-      <c r="I9" s="5">
-        <f>AVERAGE(B7:I7)</f>
-        <v>0.79231343160365375</v>
-      </c>
-      <c r="U9" s="5">
-        <f>AVERAGE(J7:U7)</f>
-        <v>0.67832376525116833</v>
-      </c>
-      <c r="W9" s="5">
-        <f>AVERAGE(I9,U9)</f>
-        <v>0.7353185984274111</v>
+      <c r="I9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="W9" s="5"/>
+    </row>
+    <row r="10" spans="1:51" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" t="s">
+        <v>77</v>
+      </c>
+      <c r="G10" t="s">
+        <v>78</v>
+      </c>
+      <c r="H10" t="s">
+        <v>79</v>
+      </c>
+      <c r="I10" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" t="s">
+        <v>81</v>
+      </c>
+      <c r="K10" t="s">
+        <v>82</v>
+      </c>
+      <c r="L10" t="s">
+        <v>83</v>
+      </c>
+      <c r="M10" t="s">
+        <v>84</v>
+      </c>
+      <c r="N10" t="s">
+        <v>85</v>
+      </c>
+      <c r="O10" t="s">
+        <v>86</v>
+      </c>
+      <c r="P10" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>88</v>
+      </c>
+      <c r="R10" t="s">
+        <v>89</v>
+      </c>
+      <c r="S10" t="s">
+        <v>90</v>
+      </c>
+      <c r="T10" t="s">
+        <v>91</v>
+      </c>
+      <c r="U10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:51" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11">
+        <v>0.86276146222643102</v>
+      </c>
+      <c r="C11">
+        <v>0.74074689803015803</v>
+      </c>
+      <c r="D11">
+        <v>0.85054928065416602</v>
+      </c>
+      <c r="E11">
+        <v>0.81814441680772598</v>
+      </c>
+      <c r="F11">
+        <v>0.79085038760443604</v>
+      </c>
+      <c r="G11">
+        <v>0.78504247080995204</v>
+      </c>
+      <c r="H11">
+        <v>0.86401203098463697</v>
+      </c>
+      <c r="I11">
+        <v>0.71166563560714802</v>
+      </c>
+      <c r="J11">
+        <v>0.81491130084522601</v>
+      </c>
+      <c r="K11">
+        <v>0.86785674397944002</v>
+      </c>
+      <c r="L11">
+        <v>0.33721816546926398</v>
+      </c>
+      <c r="M11">
+        <v>0.69365086432215095</v>
+      </c>
+      <c r="N11">
+        <v>0.68848032279059901</v>
+      </c>
+      <c r="O11">
+        <v>0.449340985843523</v>
+      </c>
+      <c r="P11">
+        <v>0.81228571162530305</v>
+      </c>
+      <c r="Q11">
+        <v>0.83411116863041002</v>
+      </c>
+      <c r="R11">
+        <v>0.64685998237570397</v>
+      </c>
+      <c r="S11">
+        <v>0.73210706007850201</v>
+      </c>
+      <c r="T11">
+        <v>0.705625661637861</v>
+      </c>
+      <c r="U11">
+        <v>0.86637849019393798</v>
+      </c>
+    </row>
+    <row r="12" spans="1:51" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12">
+        <v>0.85352349983328701</v>
+      </c>
+      <c r="C12">
+        <v>0.724798315377438</v>
+      </c>
+      <c r="D12">
+        <v>0.82777645880776596</v>
+      </c>
+      <c r="E12">
+        <v>0.82784987948012601</v>
+      </c>
+      <c r="F12">
+        <v>0.79161955238377801</v>
+      </c>
+      <c r="G12">
+        <v>0.84375318356718498</v>
+      </c>
+      <c r="H12">
+        <v>0.79807061278984004</v>
+      </c>
+      <c r="I12">
+        <v>0.64715346567446697</v>
+      </c>
+      <c r="J12">
+        <v>0.86269506552383102</v>
+      </c>
+      <c r="K12">
+        <v>0.86957035714180098</v>
+      </c>
+      <c r="L12">
+        <v>0.58038210611443397</v>
+      </c>
+      <c r="M12">
+        <v>0.59977673890186201</v>
+      </c>
+      <c r="N12">
+        <v>0.45591494839174301</v>
+      </c>
+      <c r="O12">
+        <v>0.105153463433959</v>
+      </c>
+      <c r="P12">
+        <v>0.75883908005948497</v>
+      </c>
+      <c r="Q12">
+        <v>0.77796162730809604</v>
+      </c>
+      <c r="R12">
+        <v>0.57801020824920901</v>
+      </c>
+      <c r="S12">
+        <v>0.68423457878454397</v>
+      </c>
+      <c r="T12">
+        <v>0.61375646710571996</v>
+      </c>
+      <c r="U12">
+        <v>0.76635249505233505</v>
+      </c>
+    </row>
+    <row r="13" spans="1:51" x14ac:dyDescent="0.35">
+      <c r="I13" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="U13" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="X13" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:51" x14ac:dyDescent="0.35">
+      <c r="H14" t="s">
+        <v>101</v>
+      </c>
+      <c r="I14" s="5">
+        <f>AVERAGE(B11:I11)</f>
+        <v>0.80297157284058174</v>
+      </c>
+      <c r="T14" t="s">
+        <v>101</v>
+      </c>
+      <c r="U14" s="5">
+        <f>AVERAGE(J11:U11)</f>
+        <v>0.70406887148266017</v>
+      </c>
+      <c r="W14" t="s">
+        <v>101</v>
+      </c>
+      <c r="X14" s="5">
+        <f>AVERAGE(I14,U14)</f>
+        <v>0.75352022216162096</v>
+      </c>
+    </row>
+    <row r="15" spans="1:51" x14ac:dyDescent="0.35">
+      <c r="H15" t="s">
+        <v>102</v>
+      </c>
+      <c r="I15" s="5">
+        <f>AVERAGE(B12:I12)</f>
+        <v>0.78931812098923593</v>
+      </c>
+      <c r="T15" t="s">
+        <v>102</v>
+      </c>
+      <c r="U15" s="5">
+        <f>AVERAGE(J12:U12)</f>
+        <v>0.6377205946722514</v>
+      </c>
+      <c r="W15" t="s">
+        <v>102</v>
+      </c>
+      <c r="X15" s="5">
+        <f>AVERAGE(I15,U15)</f>
+        <v>0.71351935783074372</v>
       </c>
     </row>
   </sheetData>
@@ -34114,7 +34278,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E6E884E-4278-4958-AEF6-CE3AB5C8D996}">
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.35">
@@ -34136,10 +34300,10 @@
       <c r="G1" t="s">
         <v>78</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="5" t="s">
         <v>80</v>
       </c>
       <c r="J1" t="s">
@@ -34201,10 +34365,10 @@
       <c r="G2">
         <v>0.78505091998955501</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="5">
         <v>-0.33398042471309602</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="5">
         <v>2.2800072977221301E-2</v>
       </c>
       <c r="J2">
@@ -34266,10 +34430,10 @@
       <c r="G3">
         <v>0.83794847262402505</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="5">
         <v>0.832584473541637</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="5">
         <v>0.64171827186225805</v>
       </c>
       <c r="J3">
@@ -34287,7 +34451,7 @@
       <c r="N3">
         <v>0.44227699763089001</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="5">
         <v>0.106638622511867</v>
       </c>
       <c r="P3">
@@ -34307,6 +34471,198 @@
       </c>
       <c r="U3">
         <v>0.75541379016388399</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" t="s">
+        <v>77</v>
+      </c>
+      <c r="G5" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" t="s">
+        <v>80</v>
+      </c>
+      <c r="J5" t="s">
+        <v>81</v>
+      </c>
+      <c r="K5" t="s">
+        <v>82</v>
+      </c>
+      <c r="L5" t="s">
+        <v>83</v>
+      </c>
+      <c r="M5" t="s">
+        <v>84</v>
+      </c>
+      <c r="N5" t="s">
+        <v>85</v>
+      </c>
+      <c r="O5" t="s">
+        <v>86</v>
+      </c>
+      <c r="P5" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>88</v>
+      </c>
+      <c r="R5" t="s">
+        <v>89</v>
+      </c>
+      <c r="S5" t="s">
+        <v>90</v>
+      </c>
+      <c r="T5" t="s">
+        <v>91</v>
+      </c>
+      <c r="U5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6">
+        <v>0.86276146222643102</v>
+      </c>
+      <c r="C6">
+        <v>0.74074689803015803</v>
+      </c>
+      <c r="D6">
+        <v>0.85054928065416602</v>
+      </c>
+      <c r="E6">
+        <v>0.81814441680772598</v>
+      </c>
+      <c r="F6">
+        <v>0.79085038760443604</v>
+      </c>
+      <c r="G6">
+        <v>0.78504247080995204</v>
+      </c>
+      <c r="H6">
+        <v>0.86401203098463697</v>
+      </c>
+      <c r="I6">
+        <v>0.71166563560714802</v>
+      </c>
+      <c r="J6">
+        <v>0.81491130084522601</v>
+      </c>
+      <c r="K6">
+        <v>0.86785674397944002</v>
+      </c>
+      <c r="L6">
+        <v>0.33721816546926398</v>
+      </c>
+      <c r="M6">
+        <v>0.69365086432215095</v>
+      </c>
+      <c r="N6">
+        <v>0.68848032279059901</v>
+      </c>
+      <c r="O6">
+        <v>0.449340985843523</v>
+      </c>
+      <c r="P6">
+        <v>0.81228571162530305</v>
+      </c>
+      <c r="Q6">
+        <v>0.83411116863041002</v>
+      </c>
+      <c r="R6">
+        <v>0.64685998237570397</v>
+      </c>
+      <c r="S6">
+        <v>0.73210706007850201</v>
+      </c>
+      <c r="T6">
+        <v>0.705625661637861</v>
+      </c>
+      <c r="U6">
+        <v>0.86637849019393798</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7">
+        <v>0.85352349983328701</v>
+      </c>
+      <c r="C7">
+        <v>0.724798315377438</v>
+      </c>
+      <c r="D7">
+        <v>0.82777645880776596</v>
+      </c>
+      <c r="E7">
+        <v>0.82784987948012601</v>
+      </c>
+      <c r="F7">
+        <v>0.79161955238377801</v>
+      </c>
+      <c r="G7">
+        <v>0.84375318356718498</v>
+      </c>
+      <c r="H7">
+        <v>0.79807061278984004</v>
+      </c>
+      <c r="I7">
+        <v>0.64715346567446697</v>
+      </c>
+      <c r="J7">
+        <v>0.86269506552383102</v>
+      </c>
+      <c r="K7">
+        <v>0.86957035714180098</v>
+      </c>
+      <c r="L7">
+        <v>0.58038210611443397</v>
+      </c>
+      <c r="M7">
+        <v>0.59977673890186201</v>
+      </c>
+      <c r="N7">
+        <v>0.45591494839174301</v>
+      </c>
+      <c r="O7">
+        <v>0.105153463433959</v>
+      </c>
+      <c r="P7">
+        <v>0.75883908005948497</v>
+      </c>
+      <c r="Q7">
+        <v>0.77796162730809604</v>
+      </c>
+      <c r="R7">
+        <v>0.57801020824920901</v>
+      </c>
+      <c r="S7">
+        <v>0.68423457878454397</v>
+      </c>
+      <c r="T7">
+        <v>0.61375646710571996</v>
+      </c>
+      <c r="U7">
+        <v>0.76635249505233505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed some small errors and reproduced the stats. the interrater scores for each bin size are in each file. The discrete score is not higher than the continous one. Triad 8 has a very low score (.1) for discrete, but not for continous (.4). Unsure if there is an error on this triad. After checking, all seems to be correct. This triad gives a score of 0 in NOVA. Could it be because most TE values are 0 (low)?
</commit_message>
<xml_diff>
--- a/data/annotations/TE_discrete_percentages.xlsx
+++ b/data/annotations/TE_discrete_percentages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\annotations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{FA16EFE5-F483-4B50-BE03-C341E916414E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{AF11CD2B-0494-416B-A28E-F9A75972BCAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14856" activeTab="2" xr2:uid="{8450E3AB-A0C1-455F-AE9B-DBE7A60F6C99}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14856" firstSheet="2" activeTab="2" xr2:uid="{8450E3AB-A0C1-455F-AE9B-DBE7A60F6C99}"/>
   </bookViews>
   <sheets>
     <sheet name="TE_discrete_percentages" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="112">
   <si>
     <t>task_eng</t>
   </si>
@@ -334,6 +334,33 @@
   </si>
   <si>
     <t>Discrete</t>
+  </si>
+  <si>
+    <t>.2666 .5333</t>
+  </si>
+  <si>
+    <t>.2333 .4666</t>
+  </si>
+  <si>
+    <t>avg dyads</t>
+  </si>
+  <si>
+    <t>avg triads</t>
+  </si>
+  <si>
+    <t>avg all</t>
+  </si>
+  <si>
+    <t>.2 .4</t>
+  </si>
+  <si>
+    <t>max val .6</t>
+  </si>
+  <si>
+    <t>max val .7</t>
+  </si>
+  <si>
+    <t>max val .8</t>
   </si>
 </sst>
 </file>
@@ -32450,7 +32477,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="17" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF17" t="s">
         <v>0</v>
       </c>
@@ -32529,8 +32556,17 @@
       <c r="CE17" t="s">
         <v>50</v>
       </c>
+      <c r="CG17" t="s">
+        <v>105</v>
+      </c>
+      <c r="CH17" t="s">
+        <v>106</v>
+      </c>
+      <c r="CI17" t="s">
+        <v>107</v>
+      </c>
     </row>
-    <row r="18" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="18" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF18" t="s">
         <v>63</v>
       </c>
@@ -32609,8 +32645,20 @@
       <c r="CE18">
         <v>0.11149971488310199</v>
       </c>
+      <c r="CG18">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[dyad_11_anno02]])</f>
+        <v>0.22317653602407225</v>
+      </c>
+      <c r="CH18">
+        <f>AVERAGE(Table245[[#This Row],[triad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0.23371544919232798</v>
+      </c>
+      <c r="CI18">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0.22907832739829545</v>
+      </c>
     </row>
-    <row r="19" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="19" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF19" t="s">
         <v>58</v>
       </c>
@@ -32689,8 +32737,20 @@
       <c r="CE19">
         <v>6.8561110055122595E-2</v>
       </c>
+      <c r="CG19">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[dyad_11_anno02]])</f>
+        <v>6.9687070137527743E-2</v>
+      </c>
+      <c r="CH19">
+        <f>AVERAGE(Table245[[#This Row],[triad_01_anno02]:[triad_14_anno02]])</f>
+        <v>9.4698432668246485E-2</v>
+      </c>
+      <c r="CI19">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[triad_14_anno02]])</f>
+        <v>8.369343315473024E-2</v>
+      </c>
     </row>
-    <row r="20" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="20" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF20" t="s">
         <v>56</v>
       </c>
@@ -32769,8 +32829,20 @@
       <c r="CE20">
         <v>0.112621174681619</v>
       </c>
+      <c r="CG20">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[dyad_11_anno02]])</f>
+        <v>0.10842778079815268</v>
+      </c>
+      <c r="CH20">
+        <f>AVERAGE(Table245[[#This Row],[triad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0.15155441477166101</v>
+      </c>
+      <c r="CI20">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0.13257869582331736</v>
+      </c>
     </row>
-    <row r="21" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="21" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF21" t="s">
         <v>60</v>
       </c>
@@ -32849,8 +32921,20 @@
       <c r="CE21">
         <v>0.34725337388329203</v>
       </c>
+      <c r="CG21">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[dyad_11_anno02]])</f>
+        <v>7.6465585566684119E-2</v>
+      </c>
+      <c r="CH21">
+        <f>AVERAGE(Table245[[#This Row],[triad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0.14259582684220984</v>
+      </c>
+      <c r="CI21">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0.11349852068097854</v>
+      </c>
     </row>
-    <row r="22" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="22" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF22" t="s">
         <v>57</v>
       </c>
@@ -32929,8 +33013,20 @@
       <c r="CE22">
         <v>0.13164797567002401</v>
       </c>
+      <c r="CG22">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[dyad_11_anno02]])</f>
+        <v>0.13858417753547853</v>
+      </c>
+      <c r="CH22">
+        <f>AVERAGE(Table245[[#This Row],[triad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0.14480217417267682</v>
+      </c>
+      <c r="CI22">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0.14206625565230954</v>
+      </c>
     </row>
-    <row r="23" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="23" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF23" t="s">
         <v>59</v>
       </c>
@@ -33009,8 +33105,20 @@
       <c r="CE23">
         <v>0.21199391750617699</v>
       </c>
+      <c r="CG23">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[dyad_11_anno02]])</f>
+        <v>0.21325781237195046</v>
+      </c>
+      <c r="CH23">
+        <f>AVERAGE(Table245[[#This Row],[triad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0.16035287715031482</v>
+      </c>
+      <c r="CI23">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0.18363104864783453</v>
+      </c>
     </row>
-    <row r="24" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="24" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF24" t="s">
         <v>61</v>
       </c>
@@ -33089,8 +33197,20 @@
       <c r="CE24">
         <v>0</v>
       </c>
+      <c r="CG24">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[dyad_11_anno02]])</f>
+        <v>6.8800710984991895E-2</v>
+      </c>
+      <c r="CH24">
+        <f>AVERAGE(Table245[[#This Row],[triad_01_anno02]:[triad_14_anno02]])</f>
+        <v>2.6570163231044684E-2</v>
+      </c>
+      <c r="CI24">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[triad_14_anno02]])</f>
+        <v>4.515160424278146E-2</v>
+      </c>
     </row>
-    <row r="25" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="25" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF25" t="s">
         <v>62</v>
       </c>
@@ -33169,8 +33289,20 @@
       <c r="CE25">
         <v>0</v>
       </c>
+      <c r="CG25">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[dyad_11_anno02]])</f>
+        <v>5.1645360089820173E-2</v>
+      </c>
+      <c r="CH25">
+        <f>AVERAGE(Table245[[#This Row],[triad_01_anno02]:[triad_14_anno02]])</f>
+        <v>1.0945230068736001E-5</v>
+      </c>
+      <c r="CI25">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[triad_14_anno02]])</f>
+        <v>2.2730087768359369E-2</v>
+      </c>
     </row>
-    <row r="26" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="26" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF26" t="s">
         <v>55</v>
       </c>
@@ -33249,8 +33381,20 @@
       <c r="CE26">
         <v>0</v>
       </c>
+      <c r="CG26">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[dyad_11_anno02]])</f>
+        <v>3.1286163143248728E-3</v>
+      </c>
+      <c r="CH26">
+        <f>AVERAGE(Table245[[#This Row],[triad_01_anno02]:[triad_14_anno02]])</f>
+        <v>4.3051238270361714E-4</v>
+      </c>
+      <c r="CI26">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[triad_14_anno02]])</f>
+        <v>1.6176781126169698E-3</v>
+      </c>
     </row>
-    <row r="27" spans="58:83" x14ac:dyDescent="0.35">
+    <row r="27" spans="58:87" x14ac:dyDescent="0.35">
       <c r="BF27" t="s">
         <v>54</v>
       </c>
@@ -33327,6 +33471,18 @@
         <v>0</v>
       </c>
       <c r="CE27">
+        <v>0</v>
+      </c>
+      <c r="CG27">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[dyad_11_anno02]])</f>
+        <v>0</v>
+      </c>
+      <c r="CH27">
+        <f>AVERAGE(Table245[[#This Row],[triad_01_anno02]:[triad_14_anno02]])</f>
+        <v>0</v>
+      </c>
+      <c r="CI27">
+        <f>AVERAGE(Table245[[#This Row],[dyad_01_anno02]:[triad_14_anno02]])</f>
         <v>0</v>
       </c>
     </row>
@@ -34094,19 +34250,19 @@
         <v>0.85054928065416602</v>
       </c>
       <c r="E11">
-        <v>0.81814441680772598</v>
+        <v>0.81632449232768201</v>
       </c>
       <c r="F11">
         <v>0.79085038760443604</v>
       </c>
       <c r="G11">
-        <v>0.78504247080995204</v>
+        <v>0.77813793483798299</v>
       </c>
       <c r="H11">
-        <v>0.86401203098463697</v>
+        <v>0.83075341522976798</v>
       </c>
       <c r="I11">
-        <v>0.71166563560714802</v>
+        <v>0.70869464818295702</v>
       </c>
       <c r="J11">
         <v>0.81491130084522601</v>
@@ -34115,34 +34271,34 @@
         <v>0.86785674397944002</v>
       </c>
       <c r="L11">
-        <v>0.33721816546926398</v>
+        <v>0.519005742862511</v>
       </c>
       <c r="M11">
-        <v>0.69365086432215095</v>
+        <v>0.69025879886924402</v>
       </c>
       <c r="N11">
-        <v>0.68848032279059901</v>
+        <v>0.65165587962521498</v>
       </c>
       <c r="O11">
-        <v>0.449340985843523</v>
+        <v>0.44824897491003401</v>
       </c>
       <c r="P11">
-        <v>0.81228571162530305</v>
+        <v>0.81223262502022398</v>
       </c>
       <c r="Q11">
-        <v>0.83411116863041002</v>
+        <v>0.83410906420998399</v>
       </c>
       <c r="R11">
         <v>0.64685998237570397</v>
       </c>
       <c r="S11">
-        <v>0.73210706007850201</v>
+        <v>0.73227374615366603</v>
       </c>
       <c r="T11">
-        <v>0.705625661637861</v>
+        <v>0.699216950339417</v>
       </c>
       <c r="U11">
-        <v>0.86637849019393798</v>
+        <v>0.86051623569899005</v>
       </c>
     </row>
     <row r="12" spans="1:51" x14ac:dyDescent="0.35">
@@ -34227,21 +34383,21 @@
       </c>
       <c r="I14" s="5">
         <f>AVERAGE(B11:I11)</f>
-        <v>0.80297157284058174</v>
+        <v>0.79735231488669767</v>
       </c>
       <c r="T14" t="s">
         <v>101</v>
       </c>
       <c r="U14" s="5">
         <f>AVERAGE(J11:U11)</f>
-        <v>0.70406887148266017</v>
+        <v>0.71476217040747125</v>
       </c>
       <c r="W14" t="s">
         <v>101</v>
       </c>
       <c r="X14" s="5">
         <f>AVERAGE(I14,U14)</f>
-        <v>0.75352022216162096</v>
+        <v>0.7560572426470844</v>
       </c>
     </row>
     <row r="15" spans="1:51" x14ac:dyDescent="0.35">
@@ -34278,7 +34434,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E6E884E-4278-4958-AEF6-CE3AB5C8D996}">
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.35">
@@ -34662,6 +34818,198 @@
         <v>0.61375646710571996</v>
       </c>
       <c r="U7">
+        <v>0.76635249505233505</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G9" t="s">
+        <v>78</v>
+      </c>
+      <c r="H9" t="s">
+        <v>79</v>
+      </c>
+      <c r="I9" t="s">
+        <v>80</v>
+      </c>
+      <c r="J9" t="s">
+        <v>81</v>
+      </c>
+      <c r="K9" t="s">
+        <v>82</v>
+      </c>
+      <c r="L9" t="s">
+        <v>83</v>
+      </c>
+      <c r="M9" t="s">
+        <v>84</v>
+      </c>
+      <c r="N9" t="s">
+        <v>85</v>
+      </c>
+      <c r="O9" t="s">
+        <v>86</v>
+      </c>
+      <c r="P9" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>88</v>
+      </c>
+      <c r="R9" t="s">
+        <v>89</v>
+      </c>
+      <c r="S9" t="s">
+        <v>90</v>
+      </c>
+      <c r="T9" t="s">
+        <v>91</v>
+      </c>
+      <c r="U9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10">
+        <v>0.86276146222643102</v>
+      </c>
+      <c r="C10">
+        <v>0.74074689803015803</v>
+      </c>
+      <c r="D10">
+        <v>0.85054928065416602</v>
+      </c>
+      <c r="E10">
+        <v>0.81632449232768201</v>
+      </c>
+      <c r="F10">
+        <v>0.79085038760443604</v>
+      </c>
+      <c r="G10">
+        <v>0.77813793483798299</v>
+      </c>
+      <c r="H10">
+        <v>0.83075341522976798</v>
+      </c>
+      <c r="I10">
+        <v>0.70869464818295702</v>
+      </c>
+      <c r="J10">
+        <v>0.81491130084522601</v>
+      </c>
+      <c r="K10">
+        <v>0.86785674397944002</v>
+      </c>
+      <c r="L10">
+        <v>0.519005742862511</v>
+      </c>
+      <c r="M10">
+        <v>0.69025879886924402</v>
+      </c>
+      <c r="N10">
+        <v>0.65165587962521498</v>
+      </c>
+      <c r="O10">
+        <v>0.44824897491003401</v>
+      </c>
+      <c r="P10">
+        <v>0.81223262502022398</v>
+      </c>
+      <c r="Q10">
+        <v>0.83410906420998399</v>
+      </c>
+      <c r="R10">
+        <v>0.64685998237570397</v>
+      </c>
+      <c r="S10">
+        <v>0.73227374615366603</v>
+      </c>
+      <c r="T10">
+        <v>0.699216950339417</v>
+      </c>
+      <c r="U10">
+        <v>0.86051623569899005</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11">
+        <v>0.85352349983328701</v>
+      </c>
+      <c r="C11">
+        <v>0.724798315377438</v>
+      </c>
+      <c r="D11">
+        <v>0.82777645880776596</v>
+      </c>
+      <c r="E11">
+        <v>0.82784987948012601</v>
+      </c>
+      <c r="F11">
+        <v>0.79161955238377801</v>
+      </c>
+      <c r="G11">
+        <v>0.84375318356718498</v>
+      </c>
+      <c r="H11">
+        <v>0.79807061278984004</v>
+      </c>
+      <c r="I11">
+        <v>0.64715346567446697</v>
+      </c>
+      <c r="J11">
+        <v>0.86269506552383102</v>
+      </c>
+      <c r="K11">
+        <v>0.86957035714180098</v>
+      </c>
+      <c r="L11">
+        <v>0.58038210611443397</v>
+      </c>
+      <c r="M11">
+        <v>0.59977673890186201</v>
+      </c>
+      <c r="N11">
+        <v>0.45591494839174301</v>
+      </c>
+      <c r="O11">
+        <v>0.105153463433959</v>
+      </c>
+      <c r="P11">
+        <v>0.75883908005948497</v>
+      </c>
+      <c r="Q11">
+        <v>0.77796162730809604</v>
+      </c>
+      <c r="R11">
+        <v>0.57801020824920901</v>
+      </c>
+      <c r="S11">
+        <v>0.68423457878454397</v>
+      </c>
+      <c r="T11">
+        <v>0.61375646710571996</v>
+      </c>
+      <c r="U11">
         <v>0.76635249505233505</v>
       </c>
     </row>
@@ -35343,7 +35691,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C27C4F-7112-48CC-8600-645EA3A54793}">
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:W24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -35351,7 +35699,7 @@
     <col min="12" max="12" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
         <v>73</v>
       </c>
@@ -35413,7 +35761,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>93</v>
       </c>
@@ -35478,7 +35826,7 @@
         <v>0.64309151947275001</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>94</v>
       </c>
@@ -35541,6 +35889,615 @@
       </c>
       <c r="U3">
         <v>0.77887246177411396</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E6" t="s">
+        <v>76</v>
+      </c>
+      <c r="F6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="J6" t="s">
+        <v>81</v>
+      </c>
+      <c r="K6" t="s">
+        <v>82</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M6" t="s">
+        <v>84</v>
+      </c>
+      <c r="N6" t="s">
+        <v>85</v>
+      </c>
+      <c r="O6" t="s">
+        <v>86</v>
+      </c>
+      <c r="P6" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>88</v>
+      </c>
+      <c r="R6" t="s">
+        <v>89</v>
+      </c>
+      <c r="S6" t="s">
+        <v>90</v>
+      </c>
+      <c r="T6" t="s">
+        <v>91</v>
+      </c>
+      <c r="U6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7">
+        <v>0.86276146222643102</v>
+      </c>
+      <c r="C7">
+        <v>0.74074689803015803</v>
+      </c>
+      <c r="D7">
+        <v>0.85054928065416602</v>
+      </c>
+      <c r="E7">
+        <v>0.81632449232768201</v>
+      </c>
+      <c r="F7">
+        <v>0.79085038760443604</v>
+      </c>
+      <c r="G7">
+        <v>0.77813793483798299</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0.83075341522976798</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0.70869464818295702</v>
+      </c>
+      <c r="J7">
+        <v>0.81491130084522601</v>
+      </c>
+      <c r="K7">
+        <v>0.86785674397944002</v>
+      </c>
+      <c r="L7" s="2">
+        <v>0.519005742862511</v>
+      </c>
+      <c r="M7">
+        <v>0.69025879886924402</v>
+      </c>
+      <c r="N7">
+        <v>0.65165587962521498</v>
+      </c>
+      <c r="O7">
+        <v>0.44824897491003401</v>
+      </c>
+      <c r="P7">
+        <v>0.81223262502022398</v>
+      </c>
+      <c r="Q7">
+        <v>0.83410906420998399</v>
+      </c>
+      <c r="R7">
+        <v>0.64685998237570397</v>
+      </c>
+      <c r="S7">
+        <v>0.73227374615366603</v>
+      </c>
+      <c r="T7">
+        <v>0.699216950339417</v>
+      </c>
+      <c r="U7">
+        <v>0.86051623569899005</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B8">
+        <v>0.79314388854752005</v>
+      </c>
+      <c r="C8">
+        <v>0.68072855194797</v>
+      </c>
+      <c r="D8">
+        <v>0.80705331247429002</v>
+      </c>
+      <c r="E8">
+        <v>0.83248747119794897</v>
+      </c>
+      <c r="F8">
+        <v>0.72589040915222303</v>
+      </c>
+      <c r="G8">
+        <v>0.76519008013703005</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0.81451810353786502</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0.64712438732216104</v>
+      </c>
+      <c r="J8">
+        <v>0.82549835384246695</v>
+      </c>
+      <c r="K8">
+        <v>0.84426950577799498</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0.55553431527228103</v>
+      </c>
+      <c r="M8">
+        <v>0.661630562167414</v>
+      </c>
+      <c r="N8">
+        <v>0.38786666163503603</v>
+      </c>
+      <c r="O8">
+        <v>0.10339809520130799</v>
+      </c>
+      <c r="P8">
+        <v>0.71223983573853999</v>
+      </c>
+      <c r="Q8">
+        <v>0.76989121325268495</v>
+      </c>
+      <c r="R8">
+        <v>0.38238477770825502</v>
+      </c>
+      <c r="S8">
+        <v>0.63020158794381798</v>
+      </c>
+      <c r="T8">
+        <v>0.60734894362150005</v>
+      </c>
+      <c r="U8">
+        <v>0.75178680746486903</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="C10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D10" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="D11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" t="s">
+        <v>76</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J11" t="s">
+        <v>79</v>
+      </c>
+      <c r="K11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="M11" t="s">
+        <v>82</v>
+      </c>
+      <c r="N11" t="s">
+        <v>83</v>
+      </c>
+      <c r="O11" t="s">
+        <v>84</v>
+      </c>
+      <c r="P11" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>86</v>
+      </c>
+      <c r="R11" t="s">
+        <v>87</v>
+      </c>
+      <c r="S11" t="s">
+        <v>88</v>
+      </c>
+      <c r="T11" t="s">
+        <v>89</v>
+      </c>
+      <c r="U11" t="s">
+        <v>90</v>
+      </c>
+      <c r="V11" t="s">
+        <v>91</v>
+      </c>
+      <c r="W11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="C12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12">
+        <v>0.86276146222643102</v>
+      </c>
+      <c r="E12">
+        <v>0.74074689803015803</v>
+      </c>
+      <c r="F12">
+        <v>0.85054928065416602</v>
+      </c>
+      <c r="G12">
+        <v>0.81632449232768201</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0.79085038760443604</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.77813793483798299</v>
+      </c>
+      <c r="J12">
+        <v>0.83075341522976798</v>
+      </c>
+      <c r="K12">
+        <v>0.70869464818295702</v>
+      </c>
+      <c r="L12" s="2">
+        <v>0.81491130084522601</v>
+      </c>
+      <c r="M12">
+        <v>0.86785674397944002</v>
+      </c>
+      <c r="N12">
+        <v>0.519005742862511</v>
+      </c>
+      <c r="O12">
+        <v>0.69025879886924402</v>
+      </c>
+      <c r="P12">
+        <v>0.65165587962521498</v>
+      </c>
+      <c r="Q12">
+        <v>0.44824897491003401</v>
+      </c>
+      <c r="R12">
+        <v>0.81223262502022398</v>
+      </c>
+      <c r="S12">
+        <v>0.83410906420998399</v>
+      </c>
+      <c r="T12">
+        <v>0.64685998237570397</v>
+      </c>
+      <c r="U12">
+        <v>0.73227374615366603</v>
+      </c>
+      <c r="V12">
+        <v>0.699216950339417</v>
+      </c>
+      <c r="W12">
+        <v>0.86051623569899005</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="C13" t="s">
+        <v>94</v>
+      </c>
+      <c r="D13">
+        <v>0.86162169849713799</v>
+      </c>
+      <c r="E13">
+        <v>0.75992555180224997</v>
+      </c>
+      <c r="F13">
+        <v>0.82971954888468502</v>
+      </c>
+      <c r="G13">
+        <v>0.85654398939697196</v>
+      </c>
+      <c r="H13" s="2">
+        <v>0.82473059663983705</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0.83422441088653598</v>
+      </c>
+      <c r="J13">
+        <v>0.81846720810871798</v>
+      </c>
+      <c r="K13">
+        <v>0.65046311150809499</v>
+      </c>
+      <c r="L13" s="2">
+        <v>0.89051939662495705</v>
+      </c>
+      <c r="M13">
+        <v>0.92563730644572895</v>
+      </c>
+      <c r="N13">
+        <v>0.48520127072790598</v>
+      </c>
+      <c r="O13">
+        <v>0.627092218289234</v>
+      </c>
+      <c r="P13">
+        <v>0.51003115350874895</v>
+      </c>
+      <c r="Q13">
+        <v>0.10701829802528801</v>
+      </c>
+      <c r="R13">
+        <v>0.78469907763097202</v>
+      </c>
+      <c r="S13">
+        <v>0.824431163590569</v>
+      </c>
+      <c r="T13">
+        <v>0.60443420059796604</v>
+      </c>
+      <c r="U13">
+        <v>0.68051973107670205</v>
+      </c>
+      <c r="V13">
+        <v>0.60760210890564204</v>
+      </c>
+      <c r="W13">
+        <v>0.810415670039763</v>
+      </c>
+    </row>
+    <row r="17" spans="3:23" x14ac:dyDescent="0.35">
+      <c r="Q17" s="5"/>
+    </row>
+    <row r="18" spans="3:23" x14ac:dyDescent="0.35">
+      <c r="Q18" s="5"/>
+    </row>
+    <row r="19" spans="3:23" x14ac:dyDescent="0.35">
+      <c r="Q19" s="5"/>
+    </row>
+    <row r="21" spans="3:23" x14ac:dyDescent="0.35">
+      <c r="C21" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="3:23" x14ac:dyDescent="0.35">
+      <c r="D22" t="s">
+        <v>73</v>
+      </c>
+      <c r="E22" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22" t="s">
+        <v>76</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J22" t="s">
+        <v>79</v>
+      </c>
+      <c r="K22" t="s">
+        <v>80</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="M22" t="s">
+        <v>82</v>
+      </c>
+      <c r="N22" t="s">
+        <v>83</v>
+      </c>
+      <c r="O22" t="s">
+        <v>84</v>
+      </c>
+      <c r="P22" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>86</v>
+      </c>
+      <c r="R22" t="s">
+        <v>87</v>
+      </c>
+      <c r="S22" t="s">
+        <v>88</v>
+      </c>
+      <c r="T22" t="s">
+        <v>89</v>
+      </c>
+      <c r="U22" t="s">
+        <v>90</v>
+      </c>
+      <c r="V22" t="s">
+        <v>91</v>
+      </c>
+      <c r="W22" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="23" spans="3:23" x14ac:dyDescent="0.35">
+      <c r="C23" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23">
+        <v>0.86276146222643102</v>
+      </c>
+      <c r="E23">
+        <v>0.74074689803015803</v>
+      </c>
+      <c r="F23">
+        <v>0.85054928065416602</v>
+      </c>
+      <c r="G23">
+        <v>0.81632449232768201</v>
+      </c>
+      <c r="H23" s="2">
+        <v>0.79085038760443604</v>
+      </c>
+      <c r="I23" s="2">
+        <v>0.77813793483798299</v>
+      </c>
+      <c r="J23">
+        <v>0.83075341522976798</v>
+      </c>
+      <c r="K23">
+        <v>0.70869464818295702</v>
+      </c>
+      <c r="L23" s="2">
+        <v>0.81491130084522601</v>
+      </c>
+      <c r="M23">
+        <v>0.86785674397944002</v>
+      </c>
+      <c r="N23">
+        <v>0.519005742862511</v>
+      </c>
+      <c r="O23">
+        <v>0.69025879886924402</v>
+      </c>
+      <c r="P23">
+        <v>0.65165587962521498</v>
+      </c>
+      <c r="Q23">
+        <v>0.44824897491003401</v>
+      </c>
+      <c r="R23">
+        <v>0.81223262502022398</v>
+      </c>
+      <c r="S23">
+        <v>0.83410906420998399</v>
+      </c>
+      <c r="T23">
+        <v>0.64685998237570397</v>
+      </c>
+      <c r="U23">
+        <v>0.73227374615366603</v>
+      </c>
+      <c r="V23">
+        <v>0.699216950339417</v>
+      </c>
+      <c r="W23">
+        <v>0.86051623569899005</v>
+      </c>
+    </row>
+    <row r="24" spans="3:23" x14ac:dyDescent="0.35">
+      <c r="C24" t="s">
+        <v>94</v>
+      </c>
+      <c r="D24">
+        <v>0.87329151349427903</v>
+      </c>
+      <c r="E24">
+        <v>0.80176934340182004</v>
+      </c>
+      <c r="F24">
+        <v>0.83605197895137695</v>
+      </c>
+      <c r="G24">
+        <v>0.81975662023687002</v>
+      </c>
+      <c r="H24" s="2">
+        <v>0.86323686557894896</v>
+      </c>
+      <c r="I24" s="2">
+        <v>0.812628478806532</v>
+      </c>
+      <c r="J24">
+        <v>0.82802463353703104</v>
+      </c>
+      <c r="K24">
+        <v>0.70195784309208198</v>
+      </c>
+      <c r="L24" s="2">
+        <v>0.91350308651576595</v>
+      </c>
+      <c r="M24">
+        <v>0.94134455317763999</v>
+      </c>
+      <c r="N24">
+        <v>0.52561884851548002</v>
+      </c>
+      <c r="O24">
+        <v>0.67635327187948402</v>
+      </c>
+      <c r="P24">
+        <v>0.55221033836424405</v>
+      </c>
+      <c r="Q24">
+        <v>0.11462415329616001</v>
+      </c>
+      <c r="R24">
+        <v>0.79259398999524699</v>
+      </c>
+      <c r="S24">
+        <v>0.85806510180867501</v>
+      </c>
+      <c r="T24">
+        <v>0.61135885828034597</v>
+      </c>
+      <c r="U24">
+        <v>0.71711677060452805</v>
+      </c>
+      <c r="V24">
+        <v>0.66093441773720096</v>
+      </c>
+      <c r="W24">
+        <v>0.81024684304642902</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
visuals for the bins with a max .6 for laura's annotations
</commit_message>
<xml_diff>
--- a/data/annotations/TE_discrete_percentages.xlsx
+++ b/data/annotations/TE_discrete_percentages.xlsx
@@ -8,24 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\annotations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{AF11CD2B-0494-416B-A28E-F9A75972BCAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{906A2D7E-144E-4C96-8037-F1088B3BABA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14856" firstSheet="2" activeTab="2" xr2:uid="{8450E3AB-A0C1-455F-AE9B-DBE7A60F6C99}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14856" tabRatio="666" firstSheet="2" activeTab="3" xr2:uid="{8450E3AB-A0C1-455F-AE9B-DBE7A60F6C99}"/>
   </bookViews>
   <sheets>
     <sheet name="TE_discrete_percentages" sheetId="1" r:id="rId1"/>
     <sheet name="TE_discrete_.1" sheetId="2" r:id="rId2"/>
-    <sheet name="TE_discrete_twobinsV1" sheetId="3" r:id="rId3"/>
-    <sheet name="interraterReliability windV1" sheetId="5" r:id="rId4"/>
-    <sheet name="TE_discrete_twobinsV2" sheetId="6" r:id="rId5"/>
-    <sheet name="interraterReliability windV2" sheetId="4" r:id="rId6"/>
+    <sheet name="TE_discrete_twobins_max.75" sheetId="3" r:id="rId3"/>
+    <sheet name="TE_discrete_twobins_max.6" sheetId="7" r:id="rId4"/>
+    <sheet name="interraterReliability windV1" sheetId="5" r:id="rId5"/>
+    <sheet name="TE_discrete_twobinsV2" sheetId="6" r:id="rId6"/>
+    <sheet name="interraterReliability windV2" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="112">
   <si>
     <t>task_eng</t>
   </si>
@@ -684,7 +685,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -811,6 +812,19 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color theme="1"/>
@@ -821,6 +835,37 @@
       <bottom style="thin">
         <color theme="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -868,13 +913,17 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4995,7 +5044,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>TE_discrete_twobinsV1!$A$2</c:f>
+              <c:f>TE_discrete_twobins_max.75!$A$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5021,11 +5070,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$1:$AY$1</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$1:$AY$1</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$D$1,TE_discrete_twobinsV1!$F$1,TE_discrete_twobinsV1!$H$1,TE_discrete_twobinsV1!$J$1,TE_discrete_twobinsV1!$L$1,TE_discrete_twobinsV1!$N$1,TE_discrete_twobinsV1!$T$1,TE_discrete_twobinsV1!$V$1,TE_discrete_twobinsV1!$X$1,TE_discrete_twobinsV1!$Z$1,TE_discrete_twobinsV1!$AF$1,TE_discrete_twobinsV1!$AH$1,TE_discrete_twobinsV1!$AJ$1,TE_discrete_twobinsV1!$AL$1,TE_discrete_twobinsV1!$AN$1,TE_discrete_twobinsV1!$AP$1,TE_discrete_twobinsV1!$AR$1,TE_discrete_twobinsV1!$AT$1,TE_discrete_twobinsV1!$AV$1,TE_discrete_twobinsV1!$AX$1)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$D$1,TE_discrete_twobins_max.75!$F$1,TE_discrete_twobins_max.75!$H$1,TE_discrete_twobins_max.75!$J$1,TE_discrete_twobins_max.75!$L$1,TE_discrete_twobins_max.75!$N$1,TE_discrete_twobins_max.75!$T$1,TE_discrete_twobins_max.75!$V$1,TE_discrete_twobins_max.75!$X$1,TE_discrete_twobins_max.75!$Z$1,TE_discrete_twobins_max.75!$AF$1,TE_discrete_twobins_max.75!$AH$1,TE_discrete_twobins_max.75!$AJ$1,TE_discrete_twobins_max.75!$AL$1,TE_discrete_twobins_max.75!$AN$1,TE_discrete_twobins_max.75!$AP$1,TE_discrete_twobins_max.75!$AR$1,TE_discrete_twobins_max.75!$AT$1,TE_discrete_twobins_max.75!$AV$1,TE_discrete_twobins_max.75!$AX$1)</c:f>
               <c:strCache>
                 <c:ptCount val="20"/>
                 <c:pt idx="0">
@@ -5096,11 +5145,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$2:$AY$2</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$2:$AY$2</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$D$2,TE_discrete_twobinsV1!$F$2,TE_discrete_twobinsV1!$H$2,TE_discrete_twobinsV1!$J$2,TE_discrete_twobinsV1!$L$2,TE_discrete_twobinsV1!$N$2,TE_discrete_twobinsV1!$T$2,TE_discrete_twobinsV1!$V$2,TE_discrete_twobinsV1!$X$2,TE_discrete_twobinsV1!$Z$2,TE_discrete_twobinsV1!$AF$2,TE_discrete_twobinsV1!$AH$2,TE_discrete_twobinsV1!$AJ$2,TE_discrete_twobinsV1!$AL$2,TE_discrete_twobinsV1!$AN$2,TE_discrete_twobinsV1!$AP$2,TE_discrete_twobinsV1!$AR$2,TE_discrete_twobinsV1!$AT$2,TE_discrete_twobinsV1!$AV$2,TE_discrete_twobinsV1!$AX$2)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$D$2,TE_discrete_twobins_max.75!$F$2,TE_discrete_twobins_max.75!$H$2,TE_discrete_twobins_max.75!$J$2,TE_discrete_twobins_max.75!$L$2,TE_discrete_twobins_max.75!$N$2,TE_discrete_twobins_max.75!$T$2,TE_discrete_twobins_max.75!$V$2,TE_discrete_twobins_max.75!$X$2,TE_discrete_twobins_max.75!$Z$2,TE_discrete_twobins_max.75!$AF$2,TE_discrete_twobins_max.75!$AH$2,TE_discrete_twobins_max.75!$AJ$2,TE_discrete_twobins_max.75!$AL$2,TE_discrete_twobins_max.75!$AN$2,TE_discrete_twobins_max.75!$AP$2,TE_discrete_twobins_max.75!$AR$2,TE_discrete_twobins_max.75!$AT$2,TE_discrete_twobins_max.75!$AV$2,TE_discrete_twobins_max.75!$AX$2)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -5178,7 +5227,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>TE_discrete_twobinsV1!$A$3</c:f>
+              <c:f>TE_discrete_twobins_max.75!$A$3</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5202,11 +5251,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$1:$AY$1</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$1:$AY$1</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$D$1,TE_discrete_twobinsV1!$F$1,TE_discrete_twobinsV1!$H$1,TE_discrete_twobinsV1!$J$1,TE_discrete_twobinsV1!$L$1,TE_discrete_twobinsV1!$N$1,TE_discrete_twobinsV1!$T$1,TE_discrete_twobinsV1!$V$1,TE_discrete_twobinsV1!$X$1,TE_discrete_twobinsV1!$Z$1,TE_discrete_twobinsV1!$AF$1,TE_discrete_twobinsV1!$AH$1,TE_discrete_twobinsV1!$AJ$1,TE_discrete_twobinsV1!$AL$1,TE_discrete_twobinsV1!$AN$1,TE_discrete_twobinsV1!$AP$1,TE_discrete_twobinsV1!$AR$1,TE_discrete_twobinsV1!$AT$1,TE_discrete_twobinsV1!$AV$1,TE_discrete_twobinsV1!$AX$1)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$D$1,TE_discrete_twobins_max.75!$F$1,TE_discrete_twobins_max.75!$H$1,TE_discrete_twobins_max.75!$J$1,TE_discrete_twobins_max.75!$L$1,TE_discrete_twobins_max.75!$N$1,TE_discrete_twobins_max.75!$T$1,TE_discrete_twobins_max.75!$V$1,TE_discrete_twobins_max.75!$X$1,TE_discrete_twobins_max.75!$Z$1,TE_discrete_twobins_max.75!$AF$1,TE_discrete_twobins_max.75!$AH$1,TE_discrete_twobins_max.75!$AJ$1,TE_discrete_twobins_max.75!$AL$1,TE_discrete_twobins_max.75!$AN$1,TE_discrete_twobins_max.75!$AP$1,TE_discrete_twobins_max.75!$AR$1,TE_discrete_twobins_max.75!$AT$1,TE_discrete_twobins_max.75!$AV$1,TE_discrete_twobins_max.75!$AX$1)</c:f>
               <c:strCache>
                 <c:ptCount val="20"/>
                 <c:pt idx="0">
@@ -5277,11 +5326,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$3:$AY$3</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$3:$AY$3</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$D$3,TE_discrete_twobinsV1!$F$3,TE_discrete_twobinsV1!$H$3,TE_discrete_twobinsV1!$J$3,TE_discrete_twobinsV1!$L$3,TE_discrete_twobinsV1!$N$3,TE_discrete_twobinsV1!$T$3,TE_discrete_twobinsV1!$V$3,TE_discrete_twobinsV1!$X$3,TE_discrete_twobinsV1!$Z$3,TE_discrete_twobinsV1!$AF$3,TE_discrete_twobinsV1!$AH$3,TE_discrete_twobinsV1!$AJ$3,TE_discrete_twobinsV1!$AL$3,TE_discrete_twobinsV1!$AN$3,TE_discrete_twobinsV1!$AP$3,TE_discrete_twobinsV1!$AR$3,TE_discrete_twobinsV1!$AT$3,TE_discrete_twobinsV1!$AV$3,TE_discrete_twobinsV1!$AX$3)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$D$3,TE_discrete_twobins_max.75!$F$3,TE_discrete_twobins_max.75!$H$3,TE_discrete_twobins_max.75!$J$3,TE_discrete_twobins_max.75!$L$3,TE_discrete_twobins_max.75!$N$3,TE_discrete_twobins_max.75!$T$3,TE_discrete_twobins_max.75!$V$3,TE_discrete_twobins_max.75!$X$3,TE_discrete_twobins_max.75!$Z$3,TE_discrete_twobins_max.75!$AF$3,TE_discrete_twobins_max.75!$AH$3,TE_discrete_twobins_max.75!$AJ$3,TE_discrete_twobins_max.75!$AL$3,TE_discrete_twobins_max.75!$AN$3,TE_discrete_twobins_max.75!$AP$3,TE_discrete_twobins_max.75!$AR$3,TE_discrete_twobins_max.75!$AT$3,TE_discrete_twobins_max.75!$AV$3,TE_discrete_twobins_max.75!$AX$3)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -5359,7 +5408,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>TE_discrete_twobinsV1!$A$4</c:f>
+              <c:f>TE_discrete_twobins_max.75!$A$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5383,11 +5432,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$1:$AY$1</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$1:$AY$1</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$D$1,TE_discrete_twobinsV1!$F$1,TE_discrete_twobinsV1!$H$1,TE_discrete_twobinsV1!$J$1,TE_discrete_twobinsV1!$L$1,TE_discrete_twobinsV1!$N$1,TE_discrete_twobinsV1!$T$1,TE_discrete_twobinsV1!$V$1,TE_discrete_twobinsV1!$X$1,TE_discrete_twobinsV1!$Z$1,TE_discrete_twobinsV1!$AF$1,TE_discrete_twobinsV1!$AH$1,TE_discrete_twobinsV1!$AJ$1,TE_discrete_twobinsV1!$AL$1,TE_discrete_twobinsV1!$AN$1,TE_discrete_twobinsV1!$AP$1,TE_discrete_twobinsV1!$AR$1,TE_discrete_twobinsV1!$AT$1,TE_discrete_twobinsV1!$AV$1,TE_discrete_twobinsV1!$AX$1)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$D$1,TE_discrete_twobins_max.75!$F$1,TE_discrete_twobins_max.75!$H$1,TE_discrete_twobins_max.75!$J$1,TE_discrete_twobins_max.75!$L$1,TE_discrete_twobins_max.75!$N$1,TE_discrete_twobins_max.75!$T$1,TE_discrete_twobins_max.75!$V$1,TE_discrete_twobins_max.75!$X$1,TE_discrete_twobins_max.75!$Z$1,TE_discrete_twobins_max.75!$AF$1,TE_discrete_twobins_max.75!$AH$1,TE_discrete_twobins_max.75!$AJ$1,TE_discrete_twobins_max.75!$AL$1,TE_discrete_twobins_max.75!$AN$1,TE_discrete_twobins_max.75!$AP$1,TE_discrete_twobins_max.75!$AR$1,TE_discrete_twobins_max.75!$AT$1,TE_discrete_twobins_max.75!$AV$1,TE_discrete_twobins_max.75!$AX$1)</c:f>
               <c:strCache>
                 <c:ptCount val="20"/>
                 <c:pt idx="0">
@@ -5458,11 +5507,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$4:$AY$4</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$4:$AY$4</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$D$4,TE_discrete_twobinsV1!$F$4,TE_discrete_twobinsV1!$H$4,TE_discrete_twobinsV1!$J$4,TE_discrete_twobinsV1!$L$4,TE_discrete_twobinsV1!$N$4,TE_discrete_twobinsV1!$T$4,TE_discrete_twobinsV1!$V$4,TE_discrete_twobinsV1!$X$4,TE_discrete_twobinsV1!$Z$4,TE_discrete_twobinsV1!$AF$4,TE_discrete_twobinsV1!$AH$4,TE_discrete_twobinsV1!$AJ$4,TE_discrete_twobinsV1!$AL$4,TE_discrete_twobinsV1!$AN$4,TE_discrete_twobinsV1!$AP$4,TE_discrete_twobinsV1!$AR$4,TE_discrete_twobinsV1!$AT$4,TE_discrete_twobinsV1!$AV$4,TE_discrete_twobinsV1!$AX$4)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$D$4,TE_discrete_twobins_max.75!$F$4,TE_discrete_twobins_max.75!$H$4,TE_discrete_twobins_max.75!$J$4,TE_discrete_twobins_max.75!$L$4,TE_discrete_twobins_max.75!$N$4,TE_discrete_twobins_max.75!$T$4,TE_discrete_twobins_max.75!$V$4,TE_discrete_twobins_max.75!$X$4,TE_discrete_twobins_max.75!$Z$4,TE_discrete_twobins_max.75!$AF$4,TE_discrete_twobins_max.75!$AH$4,TE_discrete_twobins_max.75!$AJ$4,TE_discrete_twobins_max.75!$AL$4,TE_discrete_twobins_max.75!$AN$4,TE_discrete_twobins_max.75!$AP$4,TE_discrete_twobins_max.75!$AR$4,TE_discrete_twobins_max.75!$AT$4,TE_discrete_twobins_max.75!$AV$4,TE_discrete_twobins_max.75!$AX$4)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -5817,7 +5866,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>TE_discrete_twobinsV1!$A$2</c:f>
+              <c:f>TE_discrete_twobins_max.75!$A$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5843,11 +5892,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$1:$AY$1</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$1:$AY$1</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$E$1,TE_discrete_twobinsV1!$G$1,TE_discrete_twobinsV1!$I$1,TE_discrete_twobinsV1!$K$1,TE_discrete_twobinsV1!$M$1,TE_discrete_twobinsV1!$O$1,TE_discrete_twobinsV1!$U$1,TE_discrete_twobinsV1!$W$1,TE_discrete_twobinsV1!$Y$1,TE_discrete_twobinsV1!$AA$1,TE_discrete_twobinsV1!$AG$1,TE_discrete_twobinsV1!$AI$1,TE_discrete_twobinsV1!$AK$1,TE_discrete_twobinsV1!$AM$1,TE_discrete_twobinsV1!$AO$1,TE_discrete_twobinsV1!$AQ$1,TE_discrete_twobinsV1!$AS$1,TE_discrete_twobinsV1!$AU$1,TE_discrete_twobinsV1!$AW$1,TE_discrete_twobinsV1!$AY$1)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$E$1,TE_discrete_twobins_max.75!$G$1,TE_discrete_twobins_max.75!$I$1,TE_discrete_twobins_max.75!$K$1,TE_discrete_twobins_max.75!$M$1,TE_discrete_twobins_max.75!$O$1,TE_discrete_twobins_max.75!$U$1,TE_discrete_twobins_max.75!$W$1,TE_discrete_twobins_max.75!$Y$1,TE_discrete_twobins_max.75!$AA$1,TE_discrete_twobins_max.75!$AG$1,TE_discrete_twobins_max.75!$AI$1,TE_discrete_twobins_max.75!$AK$1,TE_discrete_twobins_max.75!$AM$1,TE_discrete_twobins_max.75!$AO$1,TE_discrete_twobins_max.75!$AQ$1,TE_discrete_twobins_max.75!$AS$1,TE_discrete_twobins_max.75!$AU$1,TE_discrete_twobins_max.75!$AW$1,TE_discrete_twobins_max.75!$AY$1)</c:f>
               <c:strCache>
                 <c:ptCount val="20"/>
                 <c:pt idx="0">
@@ -5918,11 +5967,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$2:$AY$2</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$2:$AY$2</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$E$2,TE_discrete_twobinsV1!$G$2,TE_discrete_twobinsV1!$I$2,TE_discrete_twobinsV1!$K$2,TE_discrete_twobinsV1!$M$2,TE_discrete_twobinsV1!$O$2,TE_discrete_twobinsV1!$U$2,TE_discrete_twobinsV1!$W$2,TE_discrete_twobinsV1!$Y$2,TE_discrete_twobinsV1!$AA$2,TE_discrete_twobinsV1!$AG$2,TE_discrete_twobinsV1!$AI$2,TE_discrete_twobinsV1!$AK$2,TE_discrete_twobinsV1!$AM$2,TE_discrete_twobinsV1!$AO$2,TE_discrete_twobinsV1!$AQ$2,TE_discrete_twobinsV1!$AS$2,TE_discrete_twobinsV1!$AU$2,TE_discrete_twobinsV1!$AW$2,TE_discrete_twobinsV1!$AY$2)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$E$2,TE_discrete_twobins_max.75!$G$2,TE_discrete_twobins_max.75!$I$2,TE_discrete_twobins_max.75!$K$2,TE_discrete_twobins_max.75!$M$2,TE_discrete_twobins_max.75!$O$2,TE_discrete_twobins_max.75!$U$2,TE_discrete_twobins_max.75!$W$2,TE_discrete_twobins_max.75!$Y$2,TE_discrete_twobins_max.75!$AA$2,TE_discrete_twobins_max.75!$AG$2,TE_discrete_twobins_max.75!$AI$2,TE_discrete_twobins_max.75!$AK$2,TE_discrete_twobins_max.75!$AM$2,TE_discrete_twobins_max.75!$AO$2,TE_discrete_twobins_max.75!$AQ$2,TE_discrete_twobins_max.75!$AS$2,TE_discrete_twobins_max.75!$AU$2,TE_discrete_twobins_max.75!$AW$2,TE_discrete_twobins_max.75!$AY$2)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6000,7 +6049,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>TE_discrete_twobinsV1!$A$3</c:f>
+              <c:f>TE_discrete_twobins_max.75!$A$3</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6024,11 +6073,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$1:$AY$1</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$1:$AY$1</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$E$1,TE_discrete_twobinsV1!$G$1,TE_discrete_twobinsV1!$I$1,TE_discrete_twobinsV1!$K$1,TE_discrete_twobinsV1!$M$1,TE_discrete_twobinsV1!$O$1,TE_discrete_twobinsV1!$U$1,TE_discrete_twobinsV1!$W$1,TE_discrete_twobinsV1!$Y$1,TE_discrete_twobinsV1!$AA$1,TE_discrete_twobinsV1!$AG$1,TE_discrete_twobinsV1!$AI$1,TE_discrete_twobinsV1!$AK$1,TE_discrete_twobinsV1!$AM$1,TE_discrete_twobinsV1!$AO$1,TE_discrete_twobinsV1!$AQ$1,TE_discrete_twobinsV1!$AS$1,TE_discrete_twobinsV1!$AU$1,TE_discrete_twobinsV1!$AW$1,TE_discrete_twobinsV1!$AY$1)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$E$1,TE_discrete_twobins_max.75!$G$1,TE_discrete_twobins_max.75!$I$1,TE_discrete_twobins_max.75!$K$1,TE_discrete_twobins_max.75!$M$1,TE_discrete_twobins_max.75!$O$1,TE_discrete_twobins_max.75!$U$1,TE_discrete_twobins_max.75!$W$1,TE_discrete_twobins_max.75!$Y$1,TE_discrete_twobins_max.75!$AA$1,TE_discrete_twobins_max.75!$AG$1,TE_discrete_twobins_max.75!$AI$1,TE_discrete_twobins_max.75!$AK$1,TE_discrete_twobins_max.75!$AM$1,TE_discrete_twobins_max.75!$AO$1,TE_discrete_twobins_max.75!$AQ$1,TE_discrete_twobins_max.75!$AS$1,TE_discrete_twobins_max.75!$AU$1,TE_discrete_twobins_max.75!$AW$1,TE_discrete_twobins_max.75!$AY$1)</c:f>
               <c:strCache>
                 <c:ptCount val="20"/>
                 <c:pt idx="0">
@@ -6099,11 +6148,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$3:$AY$3</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$3:$AY$3</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$E$3,TE_discrete_twobinsV1!$G$3,TE_discrete_twobinsV1!$I$3,TE_discrete_twobinsV1!$K$3,TE_discrete_twobinsV1!$M$3,TE_discrete_twobinsV1!$O$3,TE_discrete_twobinsV1!$U$3,TE_discrete_twobinsV1!$W$3,TE_discrete_twobinsV1!$Y$3,TE_discrete_twobinsV1!$AA$3,TE_discrete_twobinsV1!$AG$3,TE_discrete_twobinsV1!$AI$3,TE_discrete_twobinsV1!$AK$3,TE_discrete_twobinsV1!$AM$3,TE_discrete_twobinsV1!$AO$3,TE_discrete_twobinsV1!$AQ$3,TE_discrete_twobinsV1!$AS$3,TE_discrete_twobinsV1!$AU$3,TE_discrete_twobinsV1!$AW$3,TE_discrete_twobinsV1!$AY$3)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$E$3,TE_discrete_twobins_max.75!$G$3,TE_discrete_twobins_max.75!$I$3,TE_discrete_twobins_max.75!$K$3,TE_discrete_twobins_max.75!$M$3,TE_discrete_twobins_max.75!$O$3,TE_discrete_twobins_max.75!$U$3,TE_discrete_twobins_max.75!$W$3,TE_discrete_twobins_max.75!$Y$3,TE_discrete_twobins_max.75!$AA$3,TE_discrete_twobins_max.75!$AG$3,TE_discrete_twobins_max.75!$AI$3,TE_discrete_twobins_max.75!$AK$3,TE_discrete_twobins_max.75!$AM$3,TE_discrete_twobins_max.75!$AO$3,TE_discrete_twobins_max.75!$AQ$3,TE_discrete_twobins_max.75!$AS$3,TE_discrete_twobins_max.75!$AU$3,TE_discrete_twobins_max.75!$AW$3,TE_discrete_twobins_max.75!$AY$3)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6181,7 +6230,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>TE_discrete_twobinsV1!$A$4</c:f>
+              <c:f>TE_discrete_twobins_max.75!$A$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6205,11 +6254,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$1:$AY$1</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$1:$AY$1</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$E$1,TE_discrete_twobinsV1!$G$1,TE_discrete_twobinsV1!$I$1,TE_discrete_twobinsV1!$K$1,TE_discrete_twobinsV1!$M$1,TE_discrete_twobinsV1!$O$1,TE_discrete_twobinsV1!$U$1,TE_discrete_twobinsV1!$W$1,TE_discrete_twobinsV1!$Y$1,TE_discrete_twobinsV1!$AA$1,TE_discrete_twobinsV1!$AG$1,TE_discrete_twobinsV1!$AI$1,TE_discrete_twobinsV1!$AK$1,TE_discrete_twobinsV1!$AM$1,TE_discrete_twobinsV1!$AO$1,TE_discrete_twobinsV1!$AQ$1,TE_discrete_twobinsV1!$AS$1,TE_discrete_twobinsV1!$AU$1,TE_discrete_twobinsV1!$AW$1,TE_discrete_twobinsV1!$AY$1)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$E$1,TE_discrete_twobins_max.75!$G$1,TE_discrete_twobins_max.75!$I$1,TE_discrete_twobins_max.75!$K$1,TE_discrete_twobins_max.75!$M$1,TE_discrete_twobins_max.75!$O$1,TE_discrete_twobins_max.75!$U$1,TE_discrete_twobins_max.75!$W$1,TE_discrete_twobins_max.75!$Y$1,TE_discrete_twobins_max.75!$AA$1,TE_discrete_twobins_max.75!$AG$1,TE_discrete_twobins_max.75!$AI$1,TE_discrete_twobins_max.75!$AK$1,TE_discrete_twobins_max.75!$AM$1,TE_discrete_twobins_max.75!$AO$1,TE_discrete_twobins_max.75!$AQ$1,TE_discrete_twobins_max.75!$AS$1,TE_discrete_twobins_max.75!$AU$1,TE_discrete_twobins_max.75!$AW$1,TE_discrete_twobins_max.75!$AY$1)</c:f>
               <c:strCache>
                 <c:ptCount val="20"/>
                 <c:pt idx="0">
@@ -6280,11 +6329,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>TE_discrete_twobinsV1!$B$4:$AY$4</c15:sqref>
+                    <c15:sqref>TE_discrete_twobins_max.75!$B$4:$AY$4</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(TE_discrete_twobinsV1!$E$4,TE_discrete_twobinsV1!$G$4,TE_discrete_twobinsV1!$I$4,TE_discrete_twobinsV1!$K$4,TE_discrete_twobinsV1!$M$4,TE_discrete_twobinsV1!$O$4,TE_discrete_twobinsV1!$U$4,TE_discrete_twobinsV1!$W$4,TE_discrete_twobinsV1!$Y$4,TE_discrete_twobinsV1!$AA$4,TE_discrete_twobinsV1!$AG$4,TE_discrete_twobinsV1!$AI$4,TE_discrete_twobinsV1!$AK$4,TE_discrete_twobinsV1!$AM$4,TE_discrete_twobinsV1!$AO$4,TE_discrete_twobinsV1!$AQ$4,TE_discrete_twobinsV1!$AS$4,TE_discrete_twobinsV1!$AU$4,TE_discrete_twobinsV1!$AW$4,TE_discrete_twobinsV1!$AY$4)</c:f>
+              <c:f>(TE_discrete_twobins_max.75!$E$4,TE_discrete_twobins_max.75!$G$4,TE_discrete_twobins_max.75!$I$4,TE_discrete_twobins_max.75!$K$4,TE_discrete_twobins_max.75!$M$4,TE_discrete_twobins_max.75!$O$4,TE_discrete_twobins_max.75!$U$4,TE_discrete_twobins_max.75!$W$4,TE_discrete_twobins_max.75!$Y$4,TE_discrete_twobins_max.75!$AA$4,TE_discrete_twobins_max.75!$AG$4,TE_discrete_twobins_max.75!$AI$4,TE_discrete_twobins_max.75!$AK$4,TE_discrete_twobins_max.75!$AM$4,TE_discrete_twobins_max.75!$AO$4,TE_discrete_twobins_max.75!$AQ$4,TE_discrete_twobins_max.75!$AS$4,TE_discrete_twobins_max.75!$AU$4,TE_discrete_twobins_max.75!$AW$4,TE_discrete_twobins_max.75!$AY$4)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6588,6 +6637,1636 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-GB"/>
+              <a:t>Anno Helen</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="percentStacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>TE_discrete_twobins_max.6!$A$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>high</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$1:$AO$1</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$B$1,TE_discrete_twobins_max.6!$D$1,TE_discrete_twobins_max.6!$F$1,TE_discrete_twobins_max.6!$H$1,TE_discrete_twobins_max.6!$J$1,TE_discrete_twobins_max.6!$L$1,TE_discrete_twobins_max.6!$N$1,TE_discrete_twobins_max.6!$P$1,TE_discrete_twobins_max.6!$R$1,TE_discrete_twobins_max.6!$T$1,TE_discrete_twobins_max.6!$V$1,TE_discrete_twobins_max.6!$X$1,TE_discrete_twobins_max.6!$Z$1,TE_discrete_twobins_max.6!$AB$1,TE_discrete_twobins_max.6!$AD$1,TE_discrete_twobins_max.6!$AF$1,TE_discrete_twobins_max.6!$AH$1,TE_discrete_twobins_max.6!$AJ$1,TE_discrete_twobins_max.6!$AL$1,TE_discrete_twobins_max.6!$AN$1)</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>dyad_02_anno01</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>dyad_03_anno01</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>dyad_04_anno01</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>dyad_05_anno01</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>dyad_06_anno01</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>dyad_07_anno01</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>dyad_10_anno01</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>dyad_11_anno01</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>triad_01_anno01</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>triad_02_anno01</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>triad_05_anno01</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>triad_06_anno01</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>triad_07_anno01</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>triad_08_anno01</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>triad_09_anno01</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>triad_10_anno01</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>triad_11_anno01</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>triad_12_anno01</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>triad_13_anno01</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>triad_14_anno01</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$2:$AO$2</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$B$2,TE_discrete_twobins_max.6!$D$2,TE_discrete_twobins_max.6!$F$2,TE_discrete_twobins_max.6!$H$2,TE_discrete_twobins_max.6!$J$2,TE_discrete_twobins_max.6!$L$2,TE_discrete_twobins_max.6!$N$2,TE_discrete_twobins_max.6!$P$2,TE_discrete_twobins_max.6!$R$2,TE_discrete_twobins_max.6!$T$2,TE_discrete_twobins_max.6!$V$2,TE_discrete_twobins_max.6!$X$2,TE_discrete_twobins_max.6!$Z$2,TE_discrete_twobins_max.6!$AB$2,TE_discrete_twobins_max.6!$AD$2,TE_discrete_twobins_max.6!$AF$2,TE_discrete_twobins_max.6!$AH$2,TE_discrete_twobins_max.6!$AJ$2,TE_discrete_twobins_max.6!$AL$2,TE_discrete_twobins_max.6!$AN$2)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.47961134477407102</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.74818318506452797</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.66684062557869395</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.43899452362325198</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.92854612515368096</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.695354742861091</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.116140428350629</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.60213659380017204</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.43328185212397402</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.79845533254624101</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.63778406624884898</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.71398762283533301</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.35741104952619301</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>6.3156048068769899E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.69235877004801305</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.32977909011373502</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.21420744199342501</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.72785443888142598</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.69873102402570397</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.55135905721345702</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-985D-4102-B2F8-1BB4EBA5FEE4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>TE_discrete_twobins_max.6!$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>mid</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$1:$AO$1</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$B$1,TE_discrete_twobins_max.6!$D$1,TE_discrete_twobins_max.6!$F$1,TE_discrete_twobins_max.6!$H$1,TE_discrete_twobins_max.6!$J$1,TE_discrete_twobins_max.6!$L$1,TE_discrete_twobins_max.6!$N$1,TE_discrete_twobins_max.6!$P$1,TE_discrete_twobins_max.6!$R$1,TE_discrete_twobins_max.6!$T$1,TE_discrete_twobins_max.6!$V$1,TE_discrete_twobins_max.6!$X$1,TE_discrete_twobins_max.6!$Z$1,TE_discrete_twobins_max.6!$AB$1,TE_discrete_twobins_max.6!$AD$1,TE_discrete_twobins_max.6!$AF$1,TE_discrete_twobins_max.6!$AH$1,TE_discrete_twobins_max.6!$AJ$1,TE_discrete_twobins_max.6!$AL$1,TE_discrete_twobins_max.6!$AN$1)</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>dyad_02_anno01</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>dyad_03_anno01</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>dyad_04_anno01</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>dyad_05_anno01</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>dyad_06_anno01</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>dyad_07_anno01</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>dyad_10_anno01</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>dyad_11_anno01</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>triad_01_anno01</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>triad_02_anno01</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>triad_05_anno01</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>triad_06_anno01</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>triad_07_anno01</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>triad_08_anno01</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>triad_09_anno01</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>triad_10_anno01</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>triad_11_anno01</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>triad_12_anno01</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>triad_13_anno01</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>triad_14_anno01</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$3:$AO$3</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$B$3,TE_discrete_twobins_max.6!$D$3,TE_discrete_twobins_max.6!$F$3,TE_discrete_twobins_max.6!$H$3,TE_discrete_twobins_max.6!$J$3,TE_discrete_twobins_max.6!$L$3,TE_discrete_twobins_max.6!$N$3,TE_discrete_twobins_max.6!$P$3,TE_discrete_twobins_max.6!$R$3,TE_discrete_twobins_max.6!$T$3,TE_discrete_twobins_max.6!$V$3,TE_discrete_twobins_max.6!$X$3,TE_discrete_twobins_max.6!$Z$3,TE_discrete_twobins_max.6!$AB$3,TE_discrete_twobins_max.6!$AD$3,TE_discrete_twobins_max.6!$AF$3,TE_discrete_twobins_max.6!$AH$3,TE_discrete_twobins_max.6!$AJ$3,TE_discrete_twobins_max.6!$AL$3,TE_discrete_twobins_max.6!$AN$3)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.14992915139110599</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.143731988472622</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.13700106058820499</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.30067349229565599</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.1044197628623201E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.110888455093544</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.22885846765290299</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.34173150549586201</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.132581607713184</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.01908697363242E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.28904012083123498</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.20964491448342201</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.218027636586549</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.15169147100961899</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.22900704872816399</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.33970363079615001</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.71232550383534199</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.20410306508731199</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.26164732215382902</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.36618513590572099</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-985D-4102-B2F8-1BB4EBA5FEE4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>TE_discrete_twobins_max.6!$A$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>low</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$1:$AO$1</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$B$1,TE_discrete_twobins_max.6!$D$1,TE_discrete_twobins_max.6!$F$1,TE_discrete_twobins_max.6!$H$1,TE_discrete_twobins_max.6!$J$1,TE_discrete_twobins_max.6!$L$1,TE_discrete_twobins_max.6!$N$1,TE_discrete_twobins_max.6!$P$1,TE_discrete_twobins_max.6!$R$1,TE_discrete_twobins_max.6!$T$1,TE_discrete_twobins_max.6!$V$1,TE_discrete_twobins_max.6!$X$1,TE_discrete_twobins_max.6!$Z$1,TE_discrete_twobins_max.6!$AB$1,TE_discrete_twobins_max.6!$AD$1,TE_discrete_twobins_max.6!$AF$1,TE_discrete_twobins_max.6!$AH$1,TE_discrete_twobins_max.6!$AJ$1,TE_discrete_twobins_max.6!$AL$1,TE_discrete_twobins_max.6!$AN$1)</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>dyad_02_anno01</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>dyad_03_anno01</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>dyad_04_anno01</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>dyad_05_anno01</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>dyad_06_anno01</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>dyad_07_anno01</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>dyad_10_anno01</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>dyad_11_anno01</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>triad_01_anno01</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>triad_02_anno01</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>triad_05_anno01</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>triad_06_anno01</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>triad_07_anno01</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>triad_08_anno01</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>triad_09_anno01</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>triad_10_anno01</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>triad_11_anno01</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>triad_12_anno01</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>triad_13_anno01</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>triad_14_anno01</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$4:$AO$4</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$B$4,TE_discrete_twobins_max.6!$D$4,TE_discrete_twobins_max.6!$F$4,TE_discrete_twobins_max.6!$H$4,TE_discrete_twobins_max.6!$J$4,TE_discrete_twobins_max.6!$L$4,TE_discrete_twobins_max.6!$N$4,TE_discrete_twobins_max.6!$P$4,TE_discrete_twobins_max.6!$R$4,TE_discrete_twobins_max.6!$T$4,TE_discrete_twobins_max.6!$V$4,TE_discrete_twobins_max.6!$X$4,TE_discrete_twobins_max.6!$Z$4,TE_discrete_twobins_max.6!$AB$4,TE_discrete_twobins_max.6!$AD$4,TE_discrete_twobins_max.6!$AF$4,TE_discrete_twobins_max.6!$AH$4,TE_discrete_twobins_max.6!$AJ$4,TE_discrete_twobins_max.6!$AL$4,TE_discrete_twobins_max.6!$AN$4)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.37045950383482101</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.108069164265129</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.19615831383310001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.25801898023742298</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.0388839108962401E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.19373952700951799</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.65381430779421501</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.6131900703964399E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.42654930950203102</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.16135379771743399</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>7.3175812919914499E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>7.6367462681243406E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.42456131388725699</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.78515248092161005</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>7.8608642353662203E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.33051727909011303</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>7.3467054171232504E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>6.8042496031261404E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3.9621653820466E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>8.2455806880821103E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-985D-4102-B2F8-1BB4EBA5FEE4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="1855509952"/>
+        <c:axId val="1855510912"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1855509952"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1855510912"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1855510912"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1855509952"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>Anno Laura</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="percentStacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>TE_discrete_twobins_max.6!$A$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>high</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$1:$AO$1</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$C$1,TE_discrete_twobins_max.6!$E$1,TE_discrete_twobins_max.6!$G$1,TE_discrete_twobins_max.6!$I$1,TE_discrete_twobins_max.6!$K$1,TE_discrete_twobins_max.6!$M$1,TE_discrete_twobins_max.6!$O$1,TE_discrete_twobins_max.6!$Q$1,TE_discrete_twobins_max.6!$S$1,TE_discrete_twobins_max.6!$U$1,TE_discrete_twobins_max.6!$W$1,TE_discrete_twobins_max.6!$Y$1,TE_discrete_twobins_max.6!$AA$1,TE_discrete_twobins_max.6!$AC$1,TE_discrete_twobins_max.6!$AE$1,TE_discrete_twobins_max.6!$AG$1,TE_discrete_twobins_max.6!$AI$1,TE_discrete_twobins_max.6!$AK$1,TE_discrete_twobins_max.6!$AM$1,TE_discrete_twobins_max.6!$AO$1)</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>dyad_02_anno02</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>dyad_03_anno02</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>dyad_04_anno02</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>dyad_05_anno02</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>dyad_06_anno02</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>dyad_07_anno02</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>dyad_10_anno02</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>dyad_11_anno02</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>triad_01_anno02</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>triad_02_anno02</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>triad_05_anno02</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>triad_06_anno02</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>triad_07_anno02</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>triad_08_anno02</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>triad_09_anno02</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>triad_10_anno02</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>triad_11_anno02</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>triad_12_anno02</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>triad_13_anno02</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>triad_14_anno02</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$2:$AO$2</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$C$2,TE_discrete_twobins_max.6!$E$2,TE_discrete_twobins_max.6!$G$2,TE_discrete_twobins_max.6!$I$2,TE_discrete_twobins_max.6!$K$2,TE_discrete_twobins_max.6!$M$2,TE_discrete_twobins_max.6!$O$2,TE_discrete_twobins_max.6!$Q$2,TE_discrete_twobins_max.6!$S$2,TE_discrete_twobins_max.6!$U$2,TE_discrete_twobins_max.6!$W$2,TE_discrete_twobins_max.6!$Y$2,TE_discrete_twobins_max.6!$AA$2,TE_discrete_twobins_max.6!$AC$2,TE_discrete_twobins_max.6!$AE$2,TE_discrete_twobins_max.6!$AG$2,TE_discrete_twobins_max.6!$AI$2,TE_discrete_twobins_max.6!$AK$2,TE_discrete_twobins_max.6!$AM$2,TE_discrete_twobins_max.6!$AO$2)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.241717460246058</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.48646786117027901</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.52275214221982702</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.35996122317085599</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.826293525599616</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.56917788104410305</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>9.9939280194303301E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7.1466798402700593E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.212697365461606</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.60706906729634003</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.68918942379472E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.28492447076028599</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>7.0496283619830902E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.50807028297068102</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.6438101487314E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.12382464281353001</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.14697016191628001</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.21199391750617699</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1047-4E72-A8E9-B5D1A5C11E8C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>TE_discrete_twobins_max.6!$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>mid</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$1:$AO$1</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$C$1,TE_discrete_twobins_max.6!$E$1,TE_discrete_twobins_max.6!$G$1,TE_discrete_twobins_max.6!$I$1,TE_discrete_twobins_max.6!$K$1,TE_discrete_twobins_max.6!$M$1,TE_discrete_twobins_max.6!$O$1,TE_discrete_twobins_max.6!$Q$1,TE_discrete_twobins_max.6!$S$1,TE_discrete_twobins_max.6!$U$1,TE_discrete_twobins_max.6!$W$1,TE_discrete_twobins_max.6!$Y$1,TE_discrete_twobins_max.6!$AA$1,TE_discrete_twobins_max.6!$AC$1,TE_discrete_twobins_max.6!$AE$1,TE_discrete_twobins_max.6!$AG$1,TE_discrete_twobins_max.6!$AI$1,TE_discrete_twobins_max.6!$AK$1,TE_discrete_twobins_max.6!$AM$1,TE_discrete_twobins_max.6!$AO$1)</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>dyad_02_anno02</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>dyad_03_anno02</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>dyad_04_anno02</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>dyad_05_anno02</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>dyad_06_anno02</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>dyad_07_anno02</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>dyad_10_anno02</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>dyad_11_anno02</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>triad_01_anno02</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>triad_02_anno02</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>triad_05_anno02</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>triad_06_anno02</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>triad_07_anno02</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>triad_08_anno02</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>triad_09_anno02</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>triad_10_anno02</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>triad_11_anno02</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>triad_12_anno02</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>triad_13_anno02</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>triad_14_anno02</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$3:$AO$3</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$C$3,TE_discrete_twobins_max.6!$E$3,TE_discrete_twobins_max.6!$G$3,TE_discrete_twobins_max.6!$I$3,TE_discrete_twobins_max.6!$K$3,TE_discrete_twobins_max.6!$M$3,TE_discrete_twobins_max.6!$O$3,TE_discrete_twobins_max.6!$Q$3,TE_discrete_twobins_max.6!$S$3,TE_discrete_twobins_max.6!$U$3,TE_discrete_twobins_max.6!$W$3,TE_discrete_twobins_max.6!$Y$3,TE_discrete_twobins_max.6!$AA$3,TE_discrete_twobins_max.6!$AC$3,TE_discrete_twobins_max.6!$AE$3,TE_discrete_twobins_max.6!$AG$3,TE_discrete_twobins_max.6!$AI$3,TE_discrete_twobins_max.6!$AK$3,TE_discrete_twobins_max.6!$AM$3,TE_discrete_twobins_max.6!$AO$3)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.24365173972695101</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.39512592406966501</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.21691554014242101</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.28138712201095201</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.123424118027047</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.255929656054036</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.22656767498343999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.68852661479560295</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.326925672129672</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.25819067296339998</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.27978680925678301</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.52822314565461603</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.13473474496181401</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.33621823923277E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.35110838696496</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.473507217847769</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.51803325551479296</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.53185981194285004</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.28960811566995698</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.50058924158905105</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-1047-4E72-A8E9-B5D1A5C11E8C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>TE_discrete_twobins_max.6!$A$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>low</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$1:$AO$1</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$C$1,TE_discrete_twobins_max.6!$E$1,TE_discrete_twobins_max.6!$G$1,TE_discrete_twobins_max.6!$I$1,TE_discrete_twobins_max.6!$K$1,TE_discrete_twobins_max.6!$M$1,TE_discrete_twobins_max.6!$O$1,TE_discrete_twobins_max.6!$Q$1,TE_discrete_twobins_max.6!$S$1,TE_discrete_twobins_max.6!$U$1,TE_discrete_twobins_max.6!$W$1,TE_discrete_twobins_max.6!$Y$1,TE_discrete_twobins_max.6!$AA$1,TE_discrete_twobins_max.6!$AC$1,TE_discrete_twobins_max.6!$AE$1,TE_discrete_twobins_max.6!$AG$1,TE_discrete_twobins_max.6!$AI$1,TE_discrete_twobins_max.6!$AK$1,TE_discrete_twobins_max.6!$AM$1,TE_discrete_twobins_max.6!$AO$1)</c:f>
+              <c:strCache>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>dyad_02_anno02</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>dyad_03_anno02</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>dyad_04_anno02</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>dyad_05_anno02</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>dyad_06_anno02</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>dyad_07_anno02</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>dyad_10_anno02</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>dyad_11_anno02</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>triad_01_anno02</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>triad_02_anno02</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>triad_05_anno02</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>triad_06_anno02</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>triad_07_anno02</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>triad_08_anno02</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>triad_09_anno02</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>triad_10_anno02</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>triad_11_anno02</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>triad_12_anno02</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>triad_13_anno02</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>triad_14_anno02</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>TE_discrete_twobins_max.6!$B$4:$AO$4</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(TE_discrete_twobins_max.6!$C$4,TE_discrete_twobins_max.6!$E$4,TE_discrete_twobins_max.6!$G$4,TE_discrete_twobins_max.6!$I$4,TE_discrete_twobins_max.6!$K$4,TE_discrete_twobins_max.6!$M$4,TE_discrete_twobins_max.6!$O$4,TE_discrete_twobins_max.6!$Q$4,TE_discrete_twobins_max.6!$S$4,TE_discrete_twobins_max.6!$U$4,TE_discrete_twobins_max.6!$W$4,TE_discrete_twobins_max.6!$Y$4,TE_discrete_twobins_max.6!$AA$4,TE_discrete_twobins_max.6!$AC$4,TE_discrete_twobins_max.6!$AE$4,TE_discrete_twobins_max.6!$AG$4,TE_discrete_twobins_max.6!$AI$4,TE_discrete_twobins_max.6!$AK$4,TE_discrete_twobins_max.6!$AM$4,TE_discrete_twobins_max.6!$AO$4)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>0.41566766379523601</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.118374890364615</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.26033231763775</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.35149154733154098</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.9990622851069998E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.16620311987147299</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.38024398321925301</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.22852085134411901</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.44551738615405301</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.13474025974025899</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.35603548549504299</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.17344081610814799</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.64189931291665603</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.96657992456360897</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.140770252324037</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.46855861767279</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.48196674448520599</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.33659787519843598</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.55623747721077998</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.27099410758410902</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-1047-4E72-A8E9-B5D1A5C11E8C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="1855509952"/>
+        <c:axId val="1855510912"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1855509952"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1855510912"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1855510912"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1855509952"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
               <a:t>Helen</a:t>
             </a:r>
           </a:p>
@@ -7370,7 +9049,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -19344,6 +21023,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors16.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors17.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -22593,6 +24352,1016 @@
 </file>
 
 <file path=xl/charts/style15.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style16.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style17.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -27644,6 +30413,85 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>911860</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>54610</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1035050</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>54610</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E0BAD38-9583-DC64-3811-B74F9C8F599C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>899160</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1026160</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{712A12D7-2452-4884-80DF-56E0858B5574}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>311150</xdr:colOff>
       <xdr:row>11</xdr:row>
@@ -28004,6 +30852,56 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{43D77003-72FC-41C3-87BD-A5FBB1AABC59}" name="Table7" displayName="Table7" ref="A1:AO4" totalsRowShown="0">
+  <autoFilter ref="A1:AO4" xr:uid="{43D77003-72FC-41C3-87BD-A5FBB1AABC59}"/>
+  <tableColumns count="41">
+    <tableColumn id="1" xr3:uid="{FC2DAC51-5BF4-45C9-8CBB-5F2E023FFCCF}" name="task_eng"/>
+    <tableColumn id="2" xr3:uid="{7F24C492-7D02-4601-866A-78BAEB88EB0E}" name="dyad_02_anno01"/>
+    <tableColumn id="3" xr3:uid="{C1891BFD-F445-460C-9E6A-6D77E0E4C621}" name="dyad_02_anno02"/>
+    <tableColumn id="4" xr3:uid="{EDC2C213-DE1A-40C2-B091-BDD51AE57624}" name="dyad_03_anno01"/>
+    <tableColumn id="5" xr3:uid="{F373B450-4B43-449F-A850-52564AD7EB64}" name="dyad_03_anno02"/>
+    <tableColumn id="6" xr3:uid="{92320449-409B-41E0-BE88-3DFE1A3A7F0F}" name="dyad_04_anno01"/>
+    <tableColumn id="7" xr3:uid="{0D6495A1-B397-4940-8D68-188FB75C6AF8}" name="dyad_04_anno02"/>
+    <tableColumn id="8" xr3:uid="{0A02E8D0-B5F5-4E42-8942-CD64D5D77461}" name="dyad_05_anno01"/>
+    <tableColumn id="9" xr3:uid="{9DBF7BE4-D471-4C34-AF7C-BD0A43B75492}" name="dyad_05_anno02"/>
+    <tableColumn id="10" xr3:uid="{3463D826-CF64-4217-BB9E-474C0F41DF2C}" name="dyad_06_anno01"/>
+    <tableColumn id="11" xr3:uid="{AC74516E-9C45-4B4B-9C48-BDE98BF69A0B}" name="dyad_06_anno02"/>
+    <tableColumn id="12" xr3:uid="{B1CF669A-71F9-4878-8832-2975ABA8BA76}" name="dyad_07_anno01"/>
+    <tableColumn id="13" xr3:uid="{618BB242-32B5-43AC-9937-6A903077CD34}" name="dyad_07_anno02"/>
+    <tableColumn id="14" xr3:uid="{E62BFD50-9ED3-4CD1-86DE-65BDFDD2DBED}" name="dyad_10_anno01"/>
+    <tableColumn id="15" xr3:uid="{A4611B9E-2E0B-45A2-98E3-1F158F067633}" name="dyad_10_anno02"/>
+    <tableColumn id="16" xr3:uid="{6A2927A9-E70A-4AA6-BD10-C29A082888AF}" name="dyad_11_anno01"/>
+    <tableColumn id="17" xr3:uid="{353C28AD-ACED-435C-BC6C-A24CC84009E3}" name="dyad_11_anno02"/>
+    <tableColumn id="18" xr3:uid="{B4F86DAA-4D88-49A7-BD94-8D6224A70E3E}" name="triad_01_anno01"/>
+    <tableColumn id="19" xr3:uid="{05B5A658-1CD0-43A7-8107-11477F3A077A}" name="triad_01_anno02"/>
+    <tableColumn id="20" xr3:uid="{D047B543-DCBC-43C6-A17F-4D02A6B6E615}" name="triad_02_anno01"/>
+    <tableColumn id="21" xr3:uid="{3D3513BC-134D-4E60-BC75-65899C48716C}" name="triad_02_anno02"/>
+    <tableColumn id="22" xr3:uid="{276B2177-F32B-4BA6-87B3-EF61C38C6190}" name="triad_05_anno01"/>
+    <tableColumn id="23" xr3:uid="{FB430E1F-00B4-439E-8EE2-B837CA136DE1}" name="triad_05_anno02"/>
+    <tableColumn id="24" xr3:uid="{8F85512B-3E23-4A86-9F51-7743819540B1}" name="triad_06_anno01"/>
+    <tableColumn id="25" xr3:uid="{320A7445-D213-4C91-90B2-16BCC7597505}" name="triad_06_anno02"/>
+    <tableColumn id="26" xr3:uid="{8F834221-57A2-463D-8571-88AB09F5E74D}" name="triad_07_anno01"/>
+    <tableColumn id="27" xr3:uid="{13D95AAE-8749-492A-9FCF-56C6FBBB50C1}" name="triad_07_anno02"/>
+    <tableColumn id="28" xr3:uid="{9ADDFE8F-058B-44D5-AAC7-7AF487B823FC}" name="triad_08_anno01"/>
+    <tableColumn id="29" xr3:uid="{4C28F3A0-3F6D-4F0B-BB67-EE72E81C1D2C}" name="triad_08_anno02"/>
+    <tableColumn id="30" xr3:uid="{417EB2B8-47EB-4A83-8411-E233DCCBB01E}" name="triad_09_anno01"/>
+    <tableColumn id="31" xr3:uid="{3A033465-C487-4DA3-BF89-ADCFDC862AA8}" name="triad_09_anno02"/>
+    <tableColumn id="32" xr3:uid="{9E9EB5C4-71CC-4295-8144-F64F0E2EE899}" name="triad_10_anno01"/>
+    <tableColumn id="33" xr3:uid="{778C1DA6-16AE-4479-8A4F-1237E19FC8B1}" name="triad_10_anno02"/>
+    <tableColumn id="34" xr3:uid="{9B1E0C4F-341B-4C9B-99DC-96EC8328A14E}" name="triad_11_anno01"/>
+    <tableColumn id="35" xr3:uid="{B8272AF2-A1AB-42B6-B4C5-FF42D12E8D41}" name="triad_11_anno02"/>
+    <tableColumn id="36" xr3:uid="{1D38FA2E-A362-4B6A-A98E-00238224768D}" name="triad_12_anno01"/>
+    <tableColumn id="37" xr3:uid="{55144FD5-9909-4DA6-B954-28292E8CBD04}" name="triad_12_anno02"/>
+    <tableColumn id="38" xr3:uid="{7EF44916-A4DB-4D81-9A99-CD3DCD3FA8C9}" name="triad_13_anno01"/>
+    <tableColumn id="39" xr3:uid="{8CA25747-C54D-4C5F-89DA-43E92FDCF4D9}" name="triad_13_anno02"/>
+    <tableColumn id="40" xr3:uid="{1606CA01-AF36-425F-94F0-7B261117F93E}" name="triad_14_anno01"/>
+    <tableColumn id="41" xr3:uid="{730869A0-3E6E-4C09-889B-DF6EDEC6B82C}" name="triad_14_anno02"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{14C2C227-83C2-456E-B0F3-DF58A3760A57}" name="Table6" displayName="Table6" ref="A1:AO4" totalsRowShown="0">
   <autoFilter ref="A1:AO4" xr:uid="{14C2C227-83C2-456E-B0F3-DF58A3760A57}"/>
   <tableColumns count="41">
@@ -32473,7 +35371,7 @@
       </c>
     </row>
     <row r="16" spans="1:108" x14ac:dyDescent="0.35">
-      <c r="BR16" s="5" t="s">
+      <c r="BR16" s="6" t="s">
         <v>64</v>
       </c>
     </row>
@@ -34160,19 +37058,19 @@
       <c r="AX4" s="3">
         <v>8.2455806880821103E-2</v>
       </c>
-      <c r="AY4" s="4">
+      <c r="AY4" s="5">
         <v>0.27099410758410902</v>
       </c>
     </row>
     <row r="8" spans="1:51" x14ac:dyDescent="0.35">
-      <c r="I8" s="5"/>
-      <c r="U8" s="5"/>
-      <c r="W8" s="5"/>
+      <c r="I8" s="6"/>
+      <c r="U8" s="6"/>
+      <c r="W8" s="6"/>
     </row>
     <row r="9" spans="1:51" x14ac:dyDescent="0.35">
-      <c r="I9" s="5"/>
-      <c r="U9" s="5"/>
-      <c r="W9" s="5"/>
+      <c r="I9" s="6"/>
+      <c r="U9" s="6"/>
+      <c r="W9" s="6"/>
     </row>
     <row r="10" spans="1:51" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
@@ -34367,13 +37265,13 @@
       </c>
     </row>
     <row r="13" spans="1:51" x14ac:dyDescent="0.35">
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="U13" s="5" t="s">
+      <c r="U13" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="X13" s="5" t="s">
+      <c r="X13" s="6" t="s">
         <v>96</v>
       </c>
     </row>
@@ -34381,21 +37279,21 @@
       <c r="H14" t="s">
         <v>101</v>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="6">
         <f>AVERAGE(B11:I11)</f>
         <v>0.79735231488669767</v>
       </c>
       <c r="T14" t="s">
         <v>101</v>
       </c>
-      <c r="U14" s="5">
+      <c r="U14" s="6">
         <f>AVERAGE(J11:U11)</f>
         <v>0.71476217040747125</v>
       </c>
       <c r="W14" t="s">
         <v>101</v>
       </c>
-      <c r="X14" s="5">
+      <c r="X14" s="6">
         <f>AVERAGE(I14,U14)</f>
         <v>0.7560572426470844</v>
       </c>
@@ -34404,21 +37302,21 @@
       <c r="H15" t="s">
         <v>102</v>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="6">
         <f>AVERAGE(B12:I12)</f>
         <v>0.78931812098923593</v>
       </c>
       <c r="T15" t="s">
         <v>102</v>
       </c>
-      <c r="U15" s="5">
+      <c r="U15" s="6">
         <f>AVERAGE(J12:U12)</f>
         <v>0.6377205946722514</v>
       </c>
       <c r="W15" t="s">
         <v>102</v>
       </c>
-      <c r="X15" s="5">
+      <c r="X15" s="6">
         <f>AVERAGE(I15,U15)</f>
         <v>0.71351935783074372</v>
       </c>
@@ -34433,6 +37331,790 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A44710D-3F52-4CD3-8D0B-15D643BAC720}">
+  <dimension ref="A1:AO15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.7265625" customWidth="1"/>
+    <col min="2" max="17" width="15.90625" customWidth="1"/>
+    <col min="18" max="41" width="15.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" t="s">
+        <v>26</v>
+      </c>
+      <c r="V1" t="s">
+        <v>31</v>
+      </c>
+      <c r="W1" t="s">
+        <v>32</v>
+      </c>
+      <c r="X1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2">
+        <v>0.47961134477407102</v>
+      </c>
+      <c r="C2">
+        <v>0.241717460246058</v>
+      </c>
+      <c r="D2">
+        <v>0.74818318506452797</v>
+      </c>
+      <c r="E2">
+        <v>0.48646786117027901</v>
+      </c>
+      <c r="F2">
+        <v>0.66684062557869395</v>
+      </c>
+      <c r="G2">
+        <v>0.52275214221982702</v>
+      </c>
+      <c r="H2">
+        <v>0.43899452362325198</v>
+      </c>
+      <c r="I2">
+        <v>0.35996122317085599</v>
+      </c>
+      <c r="J2">
+        <v>0.92854612515368096</v>
+      </c>
+      <c r="K2">
+        <v>0.826293525599616</v>
+      </c>
+      <c r="L2">
+        <v>0.695354742861091</v>
+      </c>
+      <c r="M2">
+        <v>0.56917788104410305</v>
+      </c>
+      <c r="N2">
+        <v>0.116140428350629</v>
+      </c>
+      <c r="O2">
+        <v>9.9939280194303301E-2</v>
+      </c>
+      <c r="P2">
+        <v>0.60213659380017204</v>
+      </c>
+      <c r="Q2">
+        <v>7.1466798402700593E-2</v>
+      </c>
+      <c r="R2">
+        <v>0.43328185212397402</v>
+      </c>
+      <c r="S2">
+        <v>0.212697365461606</v>
+      </c>
+      <c r="T2">
+        <v>0.79845533254624101</v>
+      </c>
+      <c r="U2">
+        <v>0.60706906729634003</v>
+      </c>
+      <c r="V2">
+        <v>0.63778406624884898</v>
+      </c>
+      <c r="W2">
+        <v>2.68918942379472E-2</v>
+      </c>
+      <c r="X2">
+        <v>0.71398762283533301</v>
+      </c>
+      <c r="Y2">
+        <v>0.28492447076028599</v>
+      </c>
+      <c r="Z2">
+        <v>0.35741104952619301</v>
+      </c>
+      <c r="AA2">
+        <v>7.0496283619830902E-2</v>
+      </c>
+      <c r="AB2">
+        <v>6.3156048068769899E-2</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <v>0.69235877004801305</v>
+      </c>
+      <c r="AE2">
+        <v>0.50807028297068102</v>
+      </c>
+      <c r="AF2">
+        <v>0.32977909011373502</v>
+      </c>
+      <c r="AG2">
+        <v>2.6438101487314E-2</v>
+      </c>
+      <c r="AH2">
+        <v>0.21420744199342501</v>
+      </c>
+      <c r="AI2">
+        <v>0</v>
+      </c>
+      <c r="AJ2">
+        <v>0.72785443888142598</v>
+      </c>
+      <c r="AK2">
+        <v>0.12382464281353001</v>
+      </c>
+      <c r="AL2">
+        <v>0.69873102402570397</v>
+      </c>
+      <c r="AM2">
+        <v>0.14697016191628001</v>
+      </c>
+      <c r="AN2">
+        <v>0.55135905721345702</v>
+      </c>
+      <c r="AO2">
+        <v>0.21199391750617699</v>
+      </c>
+    </row>
+    <row r="3" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0.14992915139110599</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0.24365173972695101</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0.143731988472622</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0.39512592406966501</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0.13700106058820499</v>
+      </c>
+      <c r="G3" s="3">
+        <v>0.21691554014242101</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0.30067349229565599</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0.28138712201095201</v>
+      </c>
+      <c r="J3" s="3">
+        <v>1.1044197628623201E-2</v>
+      </c>
+      <c r="K3" s="3">
+        <v>0.123424118027047</v>
+      </c>
+      <c r="L3" s="3">
+        <v>0.110888455093544</v>
+      </c>
+      <c r="M3" s="3">
+        <v>0.255929656054036</v>
+      </c>
+      <c r="N3" s="3">
+        <v>0.22885846765290299</v>
+      </c>
+      <c r="O3" s="3">
+        <v>0.22656767498343999</v>
+      </c>
+      <c r="P3" s="3">
+        <v>0.34173150549586201</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>0.68852661479560295</v>
+      </c>
+      <c r="R3" s="3">
+        <v>0.132581607713184</v>
+      </c>
+      <c r="S3" s="3">
+        <v>0.326925672129672</v>
+      </c>
+      <c r="T3" s="3">
+        <v>4.01908697363242E-2</v>
+      </c>
+      <c r="U3" s="3">
+        <v>0.25819067296339998</v>
+      </c>
+      <c r="V3" s="3">
+        <v>0.28904012083123498</v>
+      </c>
+      <c r="W3" s="3">
+        <v>0.27978680925678301</v>
+      </c>
+      <c r="X3" s="3">
+        <v>0.20964491448342201</v>
+      </c>
+      <c r="Y3" s="3">
+        <v>0.52822314565461603</v>
+      </c>
+      <c r="Z3" s="3">
+        <v>0.218027636586549</v>
+      </c>
+      <c r="AA3" s="3">
+        <v>0.13473474496181401</v>
+      </c>
+      <c r="AB3" s="3">
+        <v>0.15169147100961899</v>
+      </c>
+      <c r="AC3" s="3">
+        <v>1.33621823923277E-2</v>
+      </c>
+      <c r="AD3" s="3">
+        <v>0.22900704872816399</v>
+      </c>
+      <c r="AE3" s="3">
+        <v>0.35110838696496</v>
+      </c>
+      <c r="AF3" s="3">
+        <v>0.33970363079615001</v>
+      </c>
+      <c r="AG3" s="3">
+        <v>0.473507217847769</v>
+      </c>
+      <c r="AH3" s="3">
+        <v>0.71232550383534199</v>
+      </c>
+      <c r="AI3" s="3">
+        <v>0.51803325551479296</v>
+      </c>
+      <c r="AJ3" s="3">
+        <v>0.20410306508731199</v>
+      </c>
+      <c r="AK3" s="3">
+        <v>0.53185981194285004</v>
+      </c>
+      <c r="AL3" s="3">
+        <v>0.26164732215382902</v>
+      </c>
+      <c r="AM3" s="3">
+        <v>0.28960811566995698</v>
+      </c>
+      <c r="AN3" s="3">
+        <v>0.36618513590572099</v>
+      </c>
+      <c r="AO3" s="5">
+        <v>0.50058924158905105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="8">
+        <v>0.37045950383482101</v>
+      </c>
+      <c r="C4" s="8">
+        <v>0.41566766379523601</v>
+      </c>
+      <c r="D4" s="8">
+        <v>0.108069164265129</v>
+      </c>
+      <c r="E4" s="8">
+        <v>0.118374890364615</v>
+      </c>
+      <c r="F4" s="8">
+        <v>0.19615831383310001</v>
+      </c>
+      <c r="G4" s="8">
+        <v>0.26033231763775</v>
+      </c>
+      <c r="H4" s="8">
+        <v>0.25801898023742298</v>
+      </c>
+      <c r="I4" s="8">
+        <v>0.35149154733154098</v>
+      </c>
+      <c r="J4" s="8">
+        <v>6.0388839108962401E-2</v>
+      </c>
+      <c r="K4" s="8">
+        <v>4.9990622851069998E-2</v>
+      </c>
+      <c r="L4" s="8">
+        <v>0.19373952700951799</v>
+      </c>
+      <c r="M4" s="8">
+        <v>0.16620311987147299</v>
+      </c>
+      <c r="N4" s="8">
+        <v>0.65381430779421501</v>
+      </c>
+      <c r="O4" s="8">
+        <v>0.38024398321925301</v>
+      </c>
+      <c r="P4" s="8">
+        <v>5.6131900703964399E-2</v>
+      </c>
+      <c r="Q4" s="8">
+        <v>0.22852085134411901</v>
+      </c>
+      <c r="R4" s="8">
+        <v>0.42654930950203102</v>
+      </c>
+      <c r="S4" s="8">
+        <v>0.44551738615405301</v>
+      </c>
+      <c r="T4" s="8">
+        <v>0.16135379771743399</v>
+      </c>
+      <c r="U4" s="8">
+        <v>0.13474025974025899</v>
+      </c>
+      <c r="V4" s="8">
+        <v>7.3175812919914499E-2</v>
+      </c>
+      <c r="W4" s="8">
+        <v>0.35603548549504299</v>
+      </c>
+      <c r="X4" s="8">
+        <v>7.6367462681243406E-2</v>
+      </c>
+      <c r="Y4" s="8">
+        <v>0.17344081610814799</v>
+      </c>
+      <c r="Z4" s="8">
+        <v>0.42456131388725699</v>
+      </c>
+      <c r="AA4" s="8">
+        <v>0.64189931291665603</v>
+      </c>
+      <c r="AB4" s="8">
+        <v>0.78515248092161005</v>
+      </c>
+      <c r="AC4" s="8">
+        <v>0.96657992456360897</v>
+      </c>
+      <c r="AD4" s="8">
+        <v>7.8608642353662203E-2</v>
+      </c>
+      <c r="AE4" s="8">
+        <v>0.140770252324037</v>
+      </c>
+      <c r="AF4" s="8">
+        <v>0.33051727909011303</v>
+      </c>
+      <c r="AG4" s="8">
+        <v>0.46855861767279</v>
+      </c>
+      <c r="AH4" s="8">
+        <v>7.3467054171232504E-2</v>
+      </c>
+      <c r="AI4" s="8">
+        <v>0.48196674448520599</v>
+      </c>
+      <c r="AJ4" s="8">
+        <v>6.8042496031261404E-2</v>
+      </c>
+      <c r="AK4" s="8">
+        <v>0.33659787519843598</v>
+      </c>
+      <c r="AL4" s="8">
+        <v>3.9621653820466E-2</v>
+      </c>
+      <c r="AM4" s="8">
+        <v>0.55623747721077998</v>
+      </c>
+      <c r="AN4" s="8">
+        <v>8.2455806880821103E-2</v>
+      </c>
+      <c r="AO4" s="9">
+        <v>0.27099410758410902</v>
+      </c>
+    </row>
+    <row r="8" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="J8" s="2"/>
+    </row>
+    <row r="9" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B9" t="s">
+        <v>109</v>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="J9" s="2"/>
+    </row>
+    <row r="10" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="H10" t="s">
+        <v>79</v>
+      </c>
+      <c r="I10" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K10" t="s">
+        <v>82</v>
+      </c>
+      <c r="L10" t="s">
+        <v>83</v>
+      </c>
+      <c r="M10" t="s">
+        <v>84</v>
+      </c>
+      <c r="N10" t="s">
+        <v>85</v>
+      </c>
+      <c r="O10" t="s">
+        <v>86</v>
+      </c>
+      <c r="P10" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>88</v>
+      </c>
+      <c r="R10" t="s">
+        <v>89</v>
+      </c>
+      <c r="S10" t="s">
+        <v>90</v>
+      </c>
+      <c r="T10" t="s">
+        <v>91</v>
+      </c>
+      <c r="U10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11">
+        <v>0.86276146222643102</v>
+      </c>
+      <c r="C11">
+        <v>0.74074689803015803</v>
+      </c>
+      <c r="D11">
+        <v>0.85054928065416602</v>
+      </c>
+      <c r="E11">
+        <v>0.81632449232768201</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.79085038760443604</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0.77813793483798299</v>
+      </c>
+      <c r="H11">
+        <v>0.83075341522976798</v>
+      </c>
+      <c r="I11">
+        <v>0.70869464818295702</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0.81491130084522601</v>
+      </c>
+      <c r="K11">
+        <v>0.86785674397944002</v>
+      </c>
+      <c r="L11">
+        <v>0.519005742862511</v>
+      </c>
+      <c r="M11">
+        <v>0.69025879886924402</v>
+      </c>
+      <c r="N11">
+        <v>0.65165587962521498</v>
+      </c>
+      <c r="O11">
+        <v>0.44824897491003401</v>
+      </c>
+      <c r="P11">
+        <v>0.81223262502022398</v>
+      </c>
+      <c r="Q11">
+        <v>0.83410906420998399</v>
+      </c>
+      <c r="R11">
+        <v>0.64685998237570397</v>
+      </c>
+      <c r="S11">
+        <v>0.73227374615366603</v>
+      </c>
+      <c r="T11">
+        <v>0.699216950339417</v>
+      </c>
+      <c r="U11">
+        <v>0.86051623569899005</v>
+      </c>
+    </row>
+    <row r="12" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12">
+        <v>0.87329151349427903</v>
+      </c>
+      <c r="C12">
+        <v>0.80176934340182004</v>
+      </c>
+      <c r="D12">
+        <v>0.83605197895137695</v>
+      </c>
+      <c r="E12">
+        <v>0.81975662023687002</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.86323686557894896</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0.812628478806532</v>
+      </c>
+      <c r="H12">
+        <v>0.82802463353703104</v>
+      </c>
+      <c r="I12">
+        <v>0.70195784309208198</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0.91350308651576595</v>
+      </c>
+      <c r="K12">
+        <v>0.94134455317763999</v>
+      </c>
+      <c r="L12">
+        <v>0.52561884851548002</v>
+      </c>
+      <c r="M12">
+        <v>0.67635327187948402</v>
+      </c>
+      <c r="N12">
+        <v>0.55221033836424405</v>
+      </c>
+      <c r="O12">
+        <v>0.11462415329616001</v>
+      </c>
+      <c r="P12">
+        <v>0.79259398999524699</v>
+      </c>
+      <c r="Q12">
+        <v>0.85806510180867501</v>
+      </c>
+      <c r="R12">
+        <v>0.61135885828034597</v>
+      </c>
+      <c r="S12">
+        <v>0.71711677060452805</v>
+      </c>
+      <c r="T12">
+        <v>0.66093441773720096</v>
+      </c>
+      <c r="U12">
+        <v>0.81024684304642902</v>
+      </c>
+    </row>
+    <row r="13" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="I13" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="U13" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="X13" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="H14" t="s">
+        <v>101</v>
+      </c>
+      <c r="I14" s="6">
+        <f>AVERAGE(B11:I11)</f>
+        <v>0.79735231488669767</v>
+      </c>
+      <c r="T14" t="s">
+        <v>101</v>
+      </c>
+      <c r="U14" s="6">
+        <f>AVERAGE(J11:U11)</f>
+        <v>0.71476217040747125</v>
+      </c>
+      <c r="W14" t="s">
+        <v>101</v>
+      </c>
+      <c r="X14" s="6">
+        <f>AVERAGE(I14,U14)</f>
+        <v>0.7560572426470844</v>
+      </c>
+    </row>
+    <row r="15" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="H15" t="s">
+        <v>102</v>
+      </c>
+      <c r="I15" s="6">
+        <f>AVERAGE(B12:I12)</f>
+        <v>0.81708965963736746</v>
+      </c>
+      <c r="T15" t="s">
+        <v>102</v>
+      </c>
+      <c r="U15" s="6">
+        <f>AVERAGE(J12:U12)</f>
+        <v>0.68116418610176666</v>
+      </c>
+      <c r="W15" t="s">
+        <v>102</v>
+      </c>
+      <c r="X15" s="6">
+        <f>AVERAGE(I15,U15)</f>
+        <v>0.74912692286956706</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E6E884E-4278-4958-AEF6-CE3AB5C8D996}">
   <dimension ref="A1:U11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -34456,10 +38138,10 @@
       <c r="G1" t="s">
         <v>78</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="6" t="s">
         <v>80</v>
       </c>
       <c r="J1" t="s">
@@ -34521,10 +38203,10 @@
       <c r="G2">
         <v>0.78505091998955501</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="6">
         <v>-0.33398042471309602</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="6">
         <v>2.2800072977221301E-2</v>
       </c>
       <c r="J2">
@@ -34586,10 +38268,10 @@
       <c r="G3">
         <v>0.83794847262402505</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="6">
         <v>0.832584473541637</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="6">
         <v>0.64171827186225805</v>
       </c>
       <c r="J3">
@@ -34607,7 +38289,7 @@
       <c r="N3">
         <v>0.44227699763089001</v>
       </c>
-      <c r="O3" s="5">
+      <c r="O3" s="6">
         <v>0.106638622511867</v>
       </c>
       <c r="P3">
@@ -35018,7 +38700,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02421442-5A43-463D-935D-4B7C818F7F90}">
   <dimension ref="A1:AO10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -35559,13 +39241,13 @@
       <c r="K6" t="s">
         <v>82</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="6" t="s">
         <v>83</v>
       </c>
       <c r="M6" t="s">
         <v>84</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="N6" s="6" t="s">
         <v>85</v>
       </c>
       <c r="O6" s="2" t="s">
@@ -35621,13 +39303,13 @@
       <c r="K7">
         <v>0.929829114228505</v>
       </c>
-      <c r="L7" s="5">
+      <c r="L7" s="6">
         <v>0.48798560027497401</v>
       </c>
       <c r="M7">
         <v>0.644813503873365</v>
       </c>
-      <c r="N7" s="5">
+      <c r="N7" s="6">
         <v>0.53651404360751698</v>
       </c>
       <c r="O7" s="2"/>
@@ -35656,26 +39338,26 @@
       <c r="L8" s="2"/>
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.35">
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="U9" s="5" t="s">
+      <c r="U9" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="W9" s="5" t="s">
+      <c r="W9" s="6" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.35">
-      <c r="I10" s="5">
+      <c r="I10" s="6">
         <f>AVERAGE(B7:I7)</f>
         <v>0.80998678629615406</v>
       </c>
-      <c r="U10" s="5">
+      <c r="U10" s="6">
         <f>AVERAGE(J7:U7)</f>
         <v>0.71687788941630504</v>
       </c>
-      <c r="W10" s="5">
+      <c r="W10" s="6">
         <f>AVERAGE(I10,U10)</f>
         <v>0.76343233785622955</v>
       </c>
@@ -35689,7 +39371,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C27C4F-7112-48CC-8600-645EA3A54793}">
   <dimension ref="A1:W24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -35730,13 +39412,13 @@
       <c r="K1" t="s">
         <v>82</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="6" t="s">
         <v>83</v>
       </c>
       <c r="M1" t="s">
         <v>84</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="6" t="s">
         <v>85</v>
       </c>
       <c r="O1" s="2" t="s">
@@ -35795,13 +39477,13 @@
       <c r="K2">
         <v>0.86785674397944002</v>
       </c>
-      <c r="L2" s="5">
+      <c r="L2" s="6">
         <v>-8.4598923649412197E-2</v>
       </c>
       <c r="M2">
         <v>0.21799042590743101</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="6">
         <v>-8.6805497576840196E-2</v>
       </c>
       <c r="O2" s="2">
@@ -35860,13 +39542,13 @@
       <c r="K3">
         <v>0.929829114228505</v>
       </c>
-      <c r="L3" s="5">
+      <c r="L3" s="6">
         <v>0.48798560027497401</v>
       </c>
       <c r="M3">
         <v>0.644813503873365</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3" s="6">
         <v>0.53651404360751698</v>
       </c>
       <c r="O3" s="2">
@@ -36292,13 +39974,13 @@
       </c>
     </row>
     <row r="17" spans="3:23" x14ac:dyDescent="0.35">
-      <c r="Q17" s="5"/>
+      <c r="Q17" s="6"/>
     </row>
     <row r="18" spans="3:23" x14ac:dyDescent="0.35">
-      <c r="Q18" s="5"/>
+      <c r="Q18" s="6"/>
     </row>
     <row r="19" spans="3:23" x14ac:dyDescent="0.35">
-      <c r="Q19" s="5"/>
+      <c r="Q19" s="6"/>
     </row>
     <row r="21" spans="3:23" x14ac:dyDescent="0.35">
       <c r="C21" t="s">

</xml_diff>

<commit_message>
calculating the Lins Concordance Correlation Coefficient. Some parts of the code needs to be cleaned up
</commit_message>
<xml_diff>
--- a/data/annotations/TE_discrete_percentages.xlsx
+++ b/data/annotations/TE_discrete_percentages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobregeo\Documents\GitHub\vilearn_ml\data\annotations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C7569F5-656A-4921-AED8-62F2ED16A5B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE28567C-60ED-418F-AD89-6FFA4C831842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="666" activeTab="6" xr2:uid="{8450E3AB-A0C1-455F-AE9B-DBE7A60F6C99}"/>
   </bookViews>
@@ -20,6 +20,7 @@
     <sheet name="interraterReliability windV1" sheetId="5" r:id="rId5"/>
     <sheet name="TE_discrete_twobinsV2" sheetId="6" r:id="rId6"/>
     <sheet name="interraterReliability windV2" sheetId="4" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="141">
   <si>
     <t>task_eng</t>
   </si>
@@ -384,6 +385,84 @@
   </si>
   <si>
     <t>continous</t>
+  </si>
+  <si>
+    <t>2nd pass</t>
+  </si>
+  <si>
+    <t>recording time</t>
+  </si>
+  <si>
+    <t>dyad_02_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>dyad_03_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>dyad_04_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>dyad_05_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>dyad_06_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>dyad_07_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>dyad_10_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>dyad_11_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_01_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_02_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_05_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_06_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_07_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_08_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_09_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_10_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_11_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_12_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_13_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>triad_14_interrater_LinsCCC</t>
+  </si>
+  <si>
+    <t>interaction time</t>
+  </si>
+  <si>
+    <t>1pass</t>
+  </si>
+  <si>
+    <t>nova</t>
+  </si>
+  <si>
+    <t>max val .1, equal sizes</t>
   </si>
 </sst>
 </file>
@@ -947,7 +1026,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -967,6 +1046,8 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="16" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="16" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -39761,7 +39842,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20C27C4F-7112-48CC-8600-645EA3A54793}">
-  <dimension ref="A1:W31"/>
+  <dimension ref="A1:AB82"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -40771,8 +40852,1448 @@
         <v>0.59277790034791999</v>
       </c>
     </row>
+    <row r="41" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="D41" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="E41" t="s">
+        <v>109</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="42" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="D42" t="s">
+        <v>117</v>
+      </c>
+      <c r="E42" t="s">
+        <v>118</v>
+      </c>
+      <c r="F42" t="s">
+        <v>119</v>
+      </c>
+      <c r="G42" t="s">
+        <v>120</v>
+      </c>
+      <c r="H42" t="s">
+        <v>121</v>
+      </c>
+      <c r="I42" t="s">
+        <v>122</v>
+      </c>
+      <c r="J42" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="K42" t="s">
+        <v>124</v>
+      </c>
+      <c r="L42" t="s">
+        <v>125</v>
+      </c>
+      <c r="M42" t="s">
+        <v>126</v>
+      </c>
+      <c r="N42" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="O42" t="s">
+        <v>128</v>
+      </c>
+      <c r="P42" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>130</v>
+      </c>
+      <c r="R42" t="s">
+        <v>131</v>
+      </c>
+      <c r="S42" t="s">
+        <v>132</v>
+      </c>
+      <c r="T42" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="U42" t="s">
+        <v>134</v>
+      </c>
+      <c r="V42" t="s">
+        <v>135</v>
+      </c>
+      <c r="W42" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="43" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="C43" t="s">
+        <v>93</v>
+      </c>
+      <c r="D43" s="9">
+        <v>0.56695299087627804</v>
+      </c>
+      <c r="E43" s="9">
+        <v>0.29786362151490098</v>
+      </c>
+      <c r="F43" s="9">
+        <v>0.54485610409552698</v>
+      </c>
+      <c r="G43" s="9">
+        <v>0.58000858400930699</v>
+      </c>
+      <c r="H43" s="9">
+        <v>0.30292688681248198</v>
+      </c>
+      <c r="I43" s="9">
+        <v>0.42134019300679998</v>
+      </c>
+      <c r="J43" s="9">
+        <v>0.66568539532105298</v>
+      </c>
+      <c r="K43" s="9">
+        <v>0.16491538563025299</v>
+      </c>
+      <c r="L43" s="9">
+        <v>0.56408883544882205</v>
+      </c>
+      <c r="M43" s="9">
+        <v>0.48967294123562799</v>
+      </c>
+      <c r="N43" s="9">
+        <v>8.18916630910482E-2</v>
+      </c>
+      <c r="O43" s="9">
+        <v>0.183040347275708</v>
+      </c>
+      <c r="P43" s="9">
+        <v>0.28752386374973898</v>
+      </c>
+      <c r="Q43" s="9">
+        <v>0.245814331884945</v>
+      </c>
+      <c r="R43" s="9">
+        <v>0.332122520790402</v>
+      </c>
+      <c r="S43" s="9">
+        <v>0.48384258471076902</v>
+      </c>
+      <c r="T43" s="9">
+        <v>0.116744968004624</v>
+      </c>
+      <c r="U43" s="9">
+        <v>0.16268956198352</v>
+      </c>
+      <c r="V43" s="9">
+        <v>0.115483992643605</v>
+      </c>
+      <c r="W43" s="9">
+        <v>0.29621162834199899</v>
+      </c>
+    </row>
+    <row r="44" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="C44" t="s">
+        <v>94</v>
+      </c>
+      <c r="D44" s="9">
+        <v>0.77390100041473098</v>
+      </c>
+      <c r="E44" s="9">
+        <v>0.66897224519254095</v>
+      </c>
+      <c r="F44" s="9">
+        <v>0.71694249552464295</v>
+      </c>
+      <c r="G44" s="9">
+        <v>0.69287765357339803</v>
+      </c>
+      <c r="H44" s="9">
+        <v>0.75891478580969396</v>
+      </c>
+      <c r="I44" s="9">
+        <v>0.67905632713620001</v>
+      </c>
+      <c r="J44" s="9">
+        <v>0.70425628128408102</v>
+      </c>
+      <c r="K44" s="9">
+        <v>0.43613100621275802</v>
+      </c>
+      <c r="L44" s="9">
+        <v>0.83979820344496803</v>
+      </c>
+      <c r="M44" s="9">
+        <v>0.88850087146123802</v>
+      </c>
+      <c r="N44" s="9">
+        <v>0.20566570063543399</v>
+      </c>
+      <c r="O44" s="9">
+        <v>0.45592105526330101</v>
+      </c>
+      <c r="P44" s="9">
+        <v>0.306885540779189</v>
+      </c>
+      <c r="Q44" s="9">
+        <v>5.03817374526472E-2</v>
+      </c>
+      <c r="R44" s="9">
+        <v>0.65074341613959197</v>
+      </c>
+      <c r="S44" s="9">
+        <v>0.69685022599482904</v>
+      </c>
+      <c r="T44" s="9">
+        <v>0.30691285884403902</v>
+      </c>
+      <c r="U44" s="9">
+        <v>0.35494765659611599</v>
+      </c>
+      <c r="V44" s="9">
+        <v>0.28838447185198302</v>
+      </c>
+      <c r="W44" s="9">
+        <v>0.61031416354652201</v>
+      </c>
+      <c r="Z44" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="AA44" t="s">
+        <v>109</v>
+      </c>
+      <c r="AB44" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="45" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="Z45" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="46" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="J46" t="s">
+        <v>93</v>
+      </c>
+      <c r="K46" s="9">
+        <f>AVERAGE(D43:K43)</f>
+        <v>0.44306864515832511</v>
+      </c>
+      <c r="V46" t="s">
+        <v>93</v>
+      </c>
+      <c r="W46" s="9">
+        <f>AVERAGE(L43:W43)</f>
+        <v>0.2799272699300675</v>
+      </c>
+      <c r="Z46" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA46" s="9">
+        <f xml:space="preserve"> AVERAGE(K46,W46)</f>
+        <v>0.36149795754419634</v>
+      </c>
+    </row>
+    <row r="47" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="J47" t="s">
+        <v>94</v>
+      </c>
+      <c r="K47" s="9">
+        <f>AVERAGE(D44:K44)</f>
+        <v>0.67888147439350588</v>
+      </c>
+      <c r="V47" t="s">
+        <v>94</v>
+      </c>
+      <c r="W47" s="9">
+        <f>AVERAGE(L44:W44)</f>
+        <v>0.47127549183415485</v>
+      </c>
+      <c r="Z47" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA47" s="9">
+        <f xml:space="preserve"> AVERAGE(K47,W47)</f>
+        <v>0.57507848311383036</v>
+      </c>
+    </row>
+    <row r="50" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="D50" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="E50" t="s">
+        <v>109</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="51" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="D51" t="s">
+        <v>117</v>
+      </c>
+      <c r="E51" t="s">
+        <v>118</v>
+      </c>
+      <c r="F51" t="s">
+        <v>119</v>
+      </c>
+      <c r="G51" t="s">
+        <v>120</v>
+      </c>
+      <c r="H51" t="s">
+        <v>121</v>
+      </c>
+      <c r="I51" t="s">
+        <v>122</v>
+      </c>
+      <c r="J51" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="K51" t="s">
+        <v>124</v>
+      </c>
+      <c r="L51" t="s">
+        <v>125</v>
+      </c>
+      <c r="M51" t="s">
+        <v>126</v>
+      </c>
+      <c r="N51" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="O51" t="s">
+        <v>128</v>
+      </c>
+      <c r="P51" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>130</v>
+      </c>
+      <c r="R51" t="s">
+        <v>131</v>
+      </c>
+      <c r="S51" t="s">
+        <v>132</v>
+      </c>
+      <c r="T51" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="U51" t="s">
+        <v>134</v>
+      </c>
+      <c r="V51" t="s">
+        <v>135</v>
+      </c>
+      <c r="W51" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="52" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="C52" t="s">
+        <v>93</v>
+      </c>
+      <c r="D52" s="9">
+        <v>0.56695299087627804</v>
+      </c>
+      <c r="E52" s="9">
+        <v>0.29786362151490098</v>
+      </c>
+      <c r="F52" s="9">
+        <v>0.54485610409552698</v>
+      </c>
+      <c r="G52" s="9">
+        <v>0.58000858400930699</v>
+      </c>
+      <c r="H52" s="9">
+        <v>0.30292688681248198</v>
+      </c>
+      <c r="I52" s="9">
+        <v>0.42134019300679998</v>
+      </c>
+      <c r="J52" s="9">
+        <v>0.543207223798435</v>
+      </c>
+      <c r="K52" s="9">
+        <v>0.16491538563025299</v>
+      </c>
+      <c r="L52" s="9">
+        <v>0.56408883544882205</v>
+      </c>
+      <c r="M52" s="9">
+        <v>0.48967294123562799</v>
+      </c>
+      <c r="N52" s="9">
+        <v>0.109880619361216</v>
+      </c>
+      <c r="O52" s="9">
+        <v>0.183040347275708</v>
+      </c>
+      <c r="P52" s="9">
+        <v>0.28752386374973898</v>
+      </c>
+      <c r="Q52" s="9">
+        <v>0.245814331884945</v>
+      </c>
+      <c r="R52" s="9">
+        <v>0.332122520790402</v>
+      </c>
+      <c r="S52" s="9">
+        <v>0.48384258471076902</v>
+      </c>
+      <c r="T52" s="9">
+        <v>1.62192036523598E-2</v>
+      </c>
+      <c r="U52" s="9">
+        <v>0.16268956198352</v>
+      </c>
+      <c r="V52" s="9">
+        <v>0.115483992643605</v>
+      </c>
+      <c r="W52" s="9">
+        <v>0.55620123815463995</v>
+      </c>
+    </row>
+    <row r="53" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="C53" t="s">
+        <v>94</v>
+      </c>
+      <c r="D53" s="9">
+        <v>0.77390100041473098</v>
+      </c>
+      <c r="E53" s="9">
+        <v>0.66897224519254095</v>
+      </c>
+      <c r="F53" s="9">
+        <v>0.71694249552464295</v>
+      </c>
+      <c r="G53" s="9">
+        <v>0.69287765357339803</v>
+      </c>
+      <c r="H53" s="9">
+        <v>0.75891478580969396</v>
+      </c>
+      <c r="I53" s="9">
+        <v>0.67905632713620001</v>
+      </c>
+      <c r="J53" s="9">
+        <v>0.13716333267177</v>
+      </c>
+      <c r="K53" s="9">
+        <v>0.43613100621275802</v>
+      </c>
+      <c r="L53" s="9">
+        <v>0.83979820344496803</v>
+      </c>
+      <c r="M53" s="9">
+        <v>0.88850087146123802</v>
+      </c>
+      <c r="N53" s="9">
+        <v>0.20738131494357201</v>
+      </c>
+      <c r="O53" s="9">
+        <v>0.45592105526330101</v>
+      </c>
+      <c r="P53" s="9">
+        <v>0.306885540779189</v>
+      </c>
+      <c r="Q53" s="9">
+        <v>5.03817374526472E-2</v>
+      </c>
+      <c r="R53" s="9">
+        <v>0.65074341613959197</v>
+      </c>
+      <c r="S53" s="9">
+        <v>0.69685022599482904</v>
+      </c>
+      <c r="T53" s="9">
+        <v>-2.9072222080026602E-2</v>
+      </c>
+      <c r="U53" s="9">
+        <v>0.35494765659611599</v>
+      </c>
+      <c r="V53" s="9">
+        <v>0.28838447185198302</v>
+      </c>
+      <c r="W53" s="9">
+        <v>0.303794889260384</v>
+      </c>
+      <c r="Z53" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="AA53" t="s">
+        <v>109</v>
+      </c>
+      <c r="AB53" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="54" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="Z54" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="55" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="J55" t="s">
+        <v>93</v>
+      </c>
+      <c r="K55" s="9">
+        <f>AVERAGE(D52:K52)</f>
+        <v>0.42775887371799792</v>
+      </c>
+      <c r="V55" t="s">
+        <v>93</v>
+      </c>
+      <c r="W55" s="9">
+        <f>AVERAGE(L52:W52)</f>
+        <v>0.29554833674094616</v>
+      </c>
+      <c r="Z55" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA55" s="9">
+        <f xml:space="preserve"> AVERAGE(K55,W55)</f>
+        <v>0.36165360522947204</v>
+      </c>
+    </row>
+    <row r="56" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="J56" t="s">
+        <v>94</v>
+      </c>
+      <c r="K56" s="9">
+        <f>AVERAGE(D53:K53)</f>
+        <v>0.60799485581696699</v>
+      </c>
+      <c r="V56" t="s">
+        <v>94</v>
+      </c>
+      <c r="W56" s="9">
+        <f>AVERAGE(L53:W53)</f>
+        <v>0.41787643009231612</v>
+      </c>
+      <c r="Z56" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA56" s="9">
+        <f xml:space="preserve"> AVERAGE(K56,W56)</f>
+        <v>0.51293564295464156</v>
+      </c>
+    </row>
+    <row r="57" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="K57" s="9"/>
+    </row>
+    <row r="59" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="D59" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="E59" t="s">
+        <v>109</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="60" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="D60" t="s">
+        <v>117</v>
+      </c>
+      <c r="E60" t="s">
+        <v>118</v>
+      </c>
+      <c r="F60" t="s">
+        <v>119</v>
+      </c>
+      <c r="G60" t="s">
+        <v>120</v>
+      </c>
+      <c r="H60" t="s">
+        <v>121</v>
+      </c>
+      <c r="I60" t="s">
+        <v>122</v>
+      </c>
+      <c r="J60" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="K60" t="s">
+        <v>124</v>
+      </c>
+      <c r="L60" t="s">
+        <v>125</v>
+      </c>
+      <c r="M60" t="s">
+        <v>126</v>
+      </c>
+      <c r="N60" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="O60" t="s">
+        <v>128</v>
+      </c>
+      <c r="P60" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>130</v>
+      </c>
+      <c r="R60" t="s">
+        <v>131</v>
+      </c>
+      <c r="S60" t="s">
+        <v>132</v>
+      </c>
+      <c r="T60" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="U60" t="s">
+        <v>134</v>
+      </c>
+      <c r="V60" t="s">
+        <v>135</v>
+      </c>
+      <c r="W60" s="5" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="61" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="C61" t="s">
+        <v>93</v>
+      </c>
+      <c r="D61" s="9">
+        <v>0.62900527901329695</v>
+      </c>
+      <c r="E61" s="9">
+        <v>0.30888142554504899</v>
+      </c>
+      <c r="F61" s="9">
+        <v>0.61786225082377999</v>
+      </c>
+      <c r="G61" s="9">
+        <v>0.603445672836594</v>
+      </c>
+      <c r="H61" s="9">
+        <v>0.65988685245150303</v>
+      </c>
+      <c r="I61" s="9">
+        <v>0.47780984191333398</v>
+      </c>
+      <c r="J61" s="9">
+        <v>0.73981263227810101</v>
+      </c>
+      <c r="K61" s="9">
+        <v>0.26407178197488201</v>
+      </c>
+      <c r="L61" s="9">
+        <v>0.57308153521365102</v>
+      </c>
+      <c r="M61" s="9">
+        <v>0.47805368471019999</v>
+      </c>
+      <c r="N61" s="9">
+        <v>0.16601301331808399</v>
+      </c>
+      <c r="O61" s="9">
+        <v>0.40618088037582101</v>
+      </c>
+      <c r="P61" s="9">
+        <v>0.43161067379881601</v>
+      </c>
+      <c r="Q61" s="9">
+        <v>0.257048219973393</v>
+      </c>
+      <c r="R61" s="9">
+        <v>0.62840582562066205</v>
+      </c>
+      <c r="S61" s="9">
+        <v>0.52165372621942996</v>
+      </c>
+      <c r="T61" s="9">
+        <v>9.8306605260632299E-2</v>
+      </c>
+      <c r="U61" s="9">
+        <v>0.307999405627222</v>
+      </c>
+      <c r="V61" s="9">
+        <v>0.196320632255579</v>
+      </c>
+      <c r="W61" s="9">
+        <v>0.37569047584833898</v>
+      </c>
+    </row>
+    <row r="62" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="C62" t="s">
+        <v>94</v>
+      </c>
+      <c r="D62" s="9">
+        <v>0.80711792988199504</v>
+      </c>
+      <c r="E62" s="9">
+        <v>0.67626239322022197</v>
+      </c>
+      <c r="F62" s="9">
+        <v>0.77190861421301404</v>
+      </c>
+      <c r="G62" s="9">
+        <v>0.71265252093283604</v>
+      </c>
+      <c r="H62" s="9">
+        <v>0.91844360595528796</v>
+      </c>
+      <c r="I62" s="9">
+        <v>0.73184432264408505</v>
+      </c>
+      <c r="J62" s="9">
+        <v>0.77177908934774397</v>
+      </c>
+      <c r="K62" s="9">
+        <v>0.56824165287888795</v>
+      </c>
+      <c r="L62" s="9">
+        <v>0.84426599053088502</v>
+      </c>
+      <c r="M62" s="9">
+        <v>0.85954124433123602</v>
+      </c>
+      <c r="N62" s="9">
+        <v>0.26980283483985001</v>
+      </c>
+      <c r="O62" s="9">
+        <v>0.69509225118126505</v>
+      </c>
+      <c r="P62" s="9">
+        <v>0.44406689682755401</v>
+      </c>
+      <c r="Q62" s="9">
+        <v>5.5447925938649001E-2</v>
+      </c>
+      <c r="R62" s="9">
+        <v>0.85662946315966304</v>
+      </c>
+      <c r="S62" s="9">
+        <v>0.71999295837365196</v>
+      </c>
+      <c r="T62" s="9">
+        <v>0.19595881912879501</v>
+      </c>
+      <c r="U62" s="9">
+        <v>0.51041432723851399</v>
+      </c>
+      <c r="V62" s="9">
+        <v>0.40525177290240399</v>
+      </c>
+      <c r="W62" s="9">
+        <v>0.64920786975383205</v>
+      </c>
+      <c r="Z62" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="AA62" t="s">
+        <v>109</v>
+      </c>
+      <c r="AB62" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="63" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="Z63" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="64" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="Z64" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA64" s="9">
+        <f xml:space="preserve"> AVERAGE(D61:W61)</f>
+        <v>0.43705702075291847</v>
+      </c>
+    </row>
+    <row r="65" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="Z65" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA65" s="9">
+        <f xml:space="preserve"> AVERAGE(D62:W62)</f>
+        <v>0.62319612416401848</v>
+      </c>
+    </row>
+    <row r="67" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="D67" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="E67" t="s">
+        <v>109</v>
+      </c>
+      <c r="F67" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="68" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="D68" t="s">
+        <v>117</v>
+      </c>
+      <c r="E68" t="s">
+        <v>118</v>
+      </c>
+      <c r="F68" t="s">
+        <v>119</v>
+      </c>
+      <c r="G68" t="s">
+        <v>120</v>
+      </c>
+      <c r="H68" t="s">
+        <v>121</v>
+      </c>
+      <c r="I68" t="s">
+        <v>122</v>
+      </c>
+      <c r="J68" t="s">
+        <v>123</v>
+      </c>
+      <c r="K68" t="s">
+        <v>124</v>
+      </c>
+      <c r="L68" t="s">
+        <v>125</v>
+      </c>
+      <c r="M68" t="s">
+        <v>126</v>
+      </c>
+      <c r="N68" t="s">
+        <v>127</v>
+      </c>
+      <c r="O68" t="s">
+        <v>128</v>
+      </c>
+      <c r="P68" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>130</v>
+      </c>
+      <c r="R68" t="s">
+        <v>131</v>
+      </c>
+      <c r="S68" t="s">
+        <v>132</v>
+      </c>
+      <c r="T68" t="s">
+        <v>133</v>
+      </c>
+      <c r="U68" t="s">
+        <v>134</v>
+      </c>
+      <c r="V68" t="s">
+        <v>135</v>
+      </c>
+      <c r="W68" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="69" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="C69" t="s">
+        <v>93</v>
+      </c>
+      <c r="D69" s="9">
+        <v>0.62900527901329695</v>
+      </c>
+      <c r="E69" s="9">
+        <v>0.30888142554504899</v>
+      </c>
+      <c r="F69" s="9">
+        <v>0.61786225082377999</v>
+      </c>
+      <c r="G69" s="9">
+        <v>0.603445672836594</v>
+      </c>
+      <c r="H69" s="9">
+        <v>0.65988685245150303</v>
+      </c>
+      <c r="I69" s="9">
+        <v>0.47780984191333398</v>
+      </c>
+      <c r="J69" s="9">
+        <v>0.60107527981205999</v>
+      </c>
+      <c r="K69" s="9">
+        <v>0.26407178197488201</v>
+      </c>
+      <c r="L69" s="9">
+        <v>0.57308153521365102</v>
+      </c>
+      <c r="M69" s="9">
+        <v>0.47805368471019999</v>
+      </c>
+      <c r="N69" s="9">
+        <v>0.25393365984337501</v>
+      </c>
+      <c r="O69" s="9">
+        <v>0.40618088037582101</v>
+      </c>
+      <c r="P69" s="9">
+        <v>0.43161067379881601</v>
+      </c>
+      <c r="Q69" s="9">
+        <v>0.257048219973393</v>
+      </c>
+      <c r="R69" s="9">
+        <v>0.62840582562066205</v>
+      </c>
+      <c r="S69" s="9">
+        <v>0.52165372621942996</v>
+      </c>
+      <c r="T69" s="9">
+        <v>2.6280436585339399E-2</v>
+      </c>
+      <c r="U69" s="9">
+        <v>0.307999405627222</v>
+      </c>
+      <c r="V69" s="9">
+        <v>0.196320632255579</v>
+      </c>
+      <c r="W69" s="9">
+        <v>0.68482443749672695</v>
+      </c>
+    </row>
+    <row r="70" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="C70" t="s">
+        <v>94</v>
+      </c>
+      <c r="D70" s="9">
+        <v>0.80711792988199504</v>
+      </c>
+      <c r="E70" s="9">
+        <v>0.67626239322022197</v>
+      </c>
+      <c r="F70" s="9">
+        <v>0.77190861421301404</v>
+      </c>
+      <c r="G70" s="9">
+        <v>0.71265252093283604</v>
+      </c>
+      <c r="H70" s="9">
+        <v>0.91844360595528796</v>
+      </c>
+      <c r="I70" s="9">
+        <v>0.73184432264408505</v>
+      </c>
+      <c r="J70" s="9">
+        <v>0.18963729390917899</v>
+      </c>
+      <c r="K70" s="9">
+        <v>0.56824165287888795</v>
+      </c>
+      <c r="L70" s="9">
+        <v>0.84426599053088502</v>
+      </c>
+      <c r="M70" s="9">
+        <v>0.85954124433123602</v>
+      </c>
+      <c r="N70" s="9">
+        <v>0.23289743517784001</v>
+      </c>
+      <c r="O70" s="9">
+        <v>0.69509225118126505</v>
+      </c>
+      <c r="P70" s="9">
+        <v>0.44406689682755401</v>
+      </c>
+      <c r="Q70" s="9">
+        <v>5.5447925938649001E-2</v>
+      </c>
+      <c r="R70" s="9">
+        <v>0.85662946315966304</v>
+      </c>
+      <c r="S70" s="9">
+        <v>0.71999295837365196</v>
+      </c>
+      <c r="T70" s="9">
+        <v>3.7900727635926799E-2</v>
+      </c>
+      <c r="U70" s="9">
+        <v>0.51041432723851399</v>
+      </c>
+      <c r="V70" s="9">
+        <v>0.40525177290240399</v>
+      </c>
+      <c r="W70" s="9">
+        <v>0.38652694199728299</v>
+      </c>
+    </row>
+    <row r="71" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="C71" t="s">
+        <v>139</v>
+      </c>
+      <c r="J71">
+        <v>0.76</v>
+      </c>
+      <c r="L71">
+        <v>0.64</v>
+      </c>
+      <c r="N71">
+        <v>0.11</v>
+      </c>
+      <c r="O71">
+        <v>0.5</v>
+      </c>
+      <c r="T71">
+        <v>0.48</v>
+      </c>
+      <c r="W71">
+        <v>0.23</v>
+      </c>
+      <c r="Z71" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="AA71" t="s">
+        <v>109</v>
+      </c>
+      <c r="AB71" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="72" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="Z72" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="73" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="Z73" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA73" s="9">
+        <f xml:space="preserve"> AVERAGE(D70:W70)</f>
+        <v>0.57120681344651902</v>
+      </c>
+    </row>
+    <row r="74" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="Z74" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA74" s="9">
+        <f xml:space="preserve"> AVERAGE(D71:W71)</f>
+        <v>0.45333333333333331</v>
+      </c>
+    </row>
+    <row r="79" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="D79" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="E79" t="s">
+        <v>140</v>
+      </c>
+      <c r="F79" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="80" spans="3:28" x14ac:dyDescent="0.35">
+      <c r="D80" t="s">
+        <v>117</v>
+      </c>
+      <c r="E80" t="s">
+        <v>118</v>
+      </c>
+      <c r="F80" t="s">
+        <v>119</v>
+      </c>
+      <c r="G80" t="s">
+        <v>120</v>
+      </c>
+      <c r="H80" t="s">
+        <v>121</v>
+      </c>
+      <c r="I80" t="s">
+        <v>122</v>
+      </c>
+      <c r="J80" t="s">
+        <v>123</v>
+      </c>
+      <c r="K80" t="s">
+        <v>124</v>
+      </c>
+      <c r="L80" t="s">
+        <v>125</v>
+      </c>
+      <c r="M80" t="s">
+        <v>126</v>
+      </c>
+      <c r="N80" t="s">
+        <v>127</v>
+      </c>
+      <c r="O80" t="s">
+        <v>128</v>
+      </c>
+      <c r="P80" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q80" t="s">
+        <v>130</v>
+      </c>
+      <c r="R80" t="s">
+        <v>131</v>
+      </c>
+      <c r="S80" t="s">
+        <v>132</v>
+      </c>
+      <c r="T80" t="s">
+        <v>133</v>
+      </c>
+      <c r="U80" t="s">
+        <v>134</v>
+      </c>
+      <c r="V80" t="s">
+        <v>135</v>
+      </c>
+      <c r="W80" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="81" spans="3:23" x14ac:dyDescent="0.35">
+      <c r="C81" t="s">
+        <v>93</v>
+      </c>
+      <c r="D81">
+        <v>0.56695299087627804</v>
+      </c>
+      <c r="E81">
+        <v>0.29786362151490098</v>
+      </c>
+      <c r="F81">
+        <v>0.54485610409552698</v>
+      </c>
+      <c r="G81">
+        <v>0.58000858400930699</v>
+      </c>
+      <c r="H81">
+        <v>0.30292688681248198</v>
+      </c>
+      <c r="I81">
+        <v>0.42134019300679998</v>
+      </c>
+      <c r="J81">
+        <v>0.66568539532105298</v>
+      </c>
+      <c r="K81">
+        <v>0.16491538563025299</v>
+      </c>
+      <c r="L81">
+        <v>0.56408883544882205</v>
+      </c>
+      <c r="M81">
+        <v>0.48967294123562799</v>
+      </c>
+      <c r="N81">
+        <v>8.18916630910482E-2</v>
+      </c>
+      <c r="O81">
+        <v>0.183040347275708</v>
+      </c>
+      <c r="P81">
+        <v>0.28752386374973898</v>
+      </c>
+      <c r="Q81">
+        <v>0.245814331884945</v>
+      </c>
+      <c r="R81">
+        <v>0.332122520790402</v>
+      </c>
+      <c r="S81">
+        <v>0.48384258471076902</v>
+      </c>
+      <c r="T81">
+        <v>0.116744968004624</v>
+      </c>
+      <c r="U81">
+        <v>0.16268956198352</v>
+      </c>
+      <c r="V81">
+        <v>0.115483992643605</v>
+      </c>
+      <c r="W81">
+        <v>0.29621162834199899</v>
+      </c>
+    </row>
+    <row r="82" spans="3:23" x14ac:dyDescent="0.35">
+      <c r="C82" t="s">
+        <v>94</v>
+      </c>
+      <c r="D82">
+        <v>0.50202106496160004</v>
+      </c>
+      <c r="E82">
+        <v>0.25103485476759901</v>
+      </c>
+      <c r="F82">
+        <v>0.44678811890460801</v>
+      </c>
+      <c r="G82">
+        <v>0.58543792387631799</v>
+      </c>
+      <c r="H82">
+        <v>0.31813326284791799</v>
+      </c>
+      <c r="I82">
+        <v>0.37669637533626998</v>
+      </c>
+      <c r="J82">
+        <v>0.32499434272904998</v>
+      </c>
+      <c r="K82">
+        <v>0.114558396241001</v>
+      </c>
+      <c r="L82">
+        <v>0.50595291038024504</v>
+      </c>
+      <c r="M82">
+        <v>0.35430067451708502</v>
+      </c>
+      <c r="N82">
+        <v>5.9979607854705297E-2</v>
+      </c>
+      <c r="O82">
+        <v>0.183870046843114</v>
+      </c>
+      <c r="P82">
+        <v>8.9975552164238595E-2</v>
+      </c>
+      <c r="Q82">
+        <v>3.1198372952606999E-2</v>
+      </c>
+      <c r="R82">
+        <v>0.25736771559273403</v>
+      </c>
+      <c r="S82">
+        <v>0.275305969572469</v>
+      </c>
+      <c r="T82">
+        <v>-1.9828883537705799E-2</v>
+      </c>
+      <c r="U82">
+        <v>9.1069604534750104E-2</v>
+      </c>
+      <c r="V82">
+        <v>6.3801412827765205E-2</v>
+      </c>
+      <c r="W82">
+        <v>0.22815204344407</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF647019-D9D4-4DFE-844F-0A523C731963}">
+  <dimension ref="A1:U11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="10" max="10" width="12.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G9" t="s">
+        <v>78</v>
+      </c>
+      <c r="H9" t="s">
+        <v>79</v>
+      </c>
+      <c r="I9" t="s">
+        <v>80</v>
+      </c>
+      <c r="J9" t="s">
+        <v>81</v>
+      </c>
+      <c r="K9" t="s">
+        <v>82</v>
+      </c>
+      <c r="L9" t="s">
+        <v>83</v>
+      </c>
+      <c r="M9" t="s">
+        <v>84</v>
+      </c>
+      <c r="N9" t="s">
+        <v>85</v>
+      </c>
+      <c r="O9" t="s">
+        <v>86</v>
+      </c>
+      <c r="P9" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>88</v>
+      </c>
+      <c r="R9" t="s">
+        <v>89</v>
+      </c>
+      <c r="S9" t="s">
+        <v>90</v>
+      </c>
+      <c r="T9" t="s">
+        <v>91</v>
+      </c>
+      <c r="U9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10">
+        <v>0.87679832543452596</v>
+      </c>
+      <c r="C10">
+        <v>0.74424022775423404</v>
+      </c>
+      <c r="D10">
+        <v>0.87597463417352595</v>
+      </c>
+      <c r="E10">
+        <v>0.82833629475958603</v>
+      </c>
+      <c r="F10">
+        <v>0.91720469407852401</v>
+      </c>
+      <c r="G10">
+        <v>0.80825763238031001</v>
+      </c>
+      <c r="H10">
+        <v>0.75158993302107602</v>
+      </c>
+      <c r="I10">
+        <v>0.77266859787776099</v>
+      </c>
+      <c r="J10">
+        <v>0.81717182427240698</v>
+      </c>
+      <c r="K10">
+        <v>0.85712755435300403</v>
+      </c>
+      <c r="L10">
+        <v>0.43852932031233299</v>
+      </c>
+      <c r="M10">
+        <v>0.80920216285187097</v>
+      </c>
+      <c r="N10">
+        <v>0.70766956904197398</v>
+      </c>
+      <c r="O10">
+        <v>0.454974577076318</v>
+      </c>
+      <c r="P10">
+        <v>0.89698964088228295</v>
+      </c>
+      <c r="Q10">
+        <v>0.825538361689096</v>
+      </c>
+      <c r="R10">
+        <v>0.14670277351968999</v>
+      </c>
+      <c r="S10">
+        <v>0.783034824591754</v>
+      </c>
+      <c r="T10">
+        <v>0.74171046174998201</v>
+      </c>
+      <c r="U10">
+        <v>0.82417078891634499</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11">
+        <v>0.89447358124555898</v>
+      </c>
+      <c r="C11">
+        <v>0.80703612246095102</v>
+      </c>
+      <c r="D11">
+        <v>0.87195882220170196</v>
+      </c>
+      <c r="E11">
+        <v>0.83329169112988399</v>
+      </c>
+      <c r="F11">
+        <v>0.95806365625644296</v>
+      </c>
+      <c r="G11">
+        <v>0.84820340055889698</v>
+      </c>
+      <c r="H11">
+        <v>0.37780916779162199</v>
+      </c>
+      <c r="I11">
+        <v>0.79345113851506199</v>
+      </c>
+      <c r="J11">
+        <v>0.91610643778803502</v>
+      </c>
+      <c r="K11">
+        <v>0.92487997403585998</v>
+      </c>
+      <c r="L11">
+        <v>0.396526477869034</v>
+      </c>
+      <c r="M11">
+        <v>0.84578998283020901</v>
+      </c>
+      <c r="N11">
+        <v>0.66243418353207095</v>
+      </c>
+      <c r="O11">
+        <v>0.117994272287108</v>
+      </c>
+      <c r="P11">
+        <v>0.92411657208375597</v>
+      </c>
+      <c r="Q11">
+        <v>0.86336986893276402</v>
+      </c>
+      <c r="R11">
+        <v>8.7706314257473605E-2</v>
+      </c>
+      <c r="S11">
+        <v>0.80336372219964802</v>
+      </c>
+      <c r="T11">
+        <v>0.74757396492422601</v>
+      </c>
+      <c r="U11">
+        <v>0.65924843795771004</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>